<commit_message>
Integrate screenshot evidence workflow
</commit_message>
<xml_diff>
--- a/skill/assets/ga4_tracking_plan_template.xlsx
+++ b/skill/assets/ga4_tracking_plan_template.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 GTM Protocol'!$A$3:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Parameter Reference'!$A$3:$I$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Event Matrix'!$A$5:$J$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Event Matrix'!$A$5:$F$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Screenshot Register'!$A$3:$H$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05 QA Cases'!$A$3:$I$9</definedName>
   </definedNames>
@@ -317,11 +317,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00EAF3EA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00EAF6F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF6D8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -335,7 +349,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFF6D8"/>
+          <fgColor rgb="00F4F6F8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -718,7 +732,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GA4 Tracking Plan Template</t>
+          <t>Generic GA4 ecommerce homepage tracking plan</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -765,7 +779,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>GA4 Tracking Plan Template</t>
+          <t>Generic GA4 ecommerce homepage tracking plan</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -783,9 +797,10 @@
           <t>Last update</t>
         </is>
       </c>
-      <c r="F4" s="6">
-        <f>TODAY()</f>
-        <v/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
       </c>
       <c r="G4" s="7" t="inlineStr"/>
       <c r="H4" s="8" t="inlineStr"/>
@@ -798,7 +813,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>vNext</t>
+          <t>v0.1</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -941,7 +956,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Main tracking plan: events, parameters, values, and test status.</t>
+          <t>Main tracking plan: events, parameters, and value rules.</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr"/>
@@ -963,7 +978,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Screenshot links for page and interaction evidence.</t>
+          <t>Capture requirements and visual evidence for later recette.</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr"/>
@@ -1051,12 +1066,13 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>vNext</t>
-        </is>
-      </c>
-      <c r="B18" s="16">
-        <f>TODAY()</f>
-        <v/>
+          <t>v0.1</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
@@ -1193,12 +1209,12 @@
       <c r="C5" s="18" t="inlineStr">
         <is>
           <t>window.dataLayer = window.dataLayer || [];
-dataLayer.push({ event: "event_name" });</t>
+dataLayer.push({ event: "add_to_cart" });</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>The Event Matrix lists the exact event and parameter values.</t>
+          <t>In the dataLayer object, the GTM trigger key is event. GA4 event_name is the GA4 tag setting/payload name.</t>
         </is>
       </c>
     </row>
@@ -1271,25 +1287,25 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>Matrix status</t>
+          <t>QA status</t>
         </is>
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>Record testing status as OK, KO, or Cannot test.</t>
+          <t>Record execution status in QA Cases or Screenshot Register, not inside the Event Matrix.</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>OK / KO / Cannot test</t>
+          <t>OK / KO / Cannot test / captured</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Status columns sit directly after each event value column.</t>
+          <t>Keep the Event Matrix focused on implementation rules.</t>
         </is>
       </c>
     </row>
@@ -2264,19 +2280,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -2290,10 +2302,6 @@
       <c r="D1" s="18" t="n"/>
       <c r="E1" s="18" t="n"/>
       <c r="F1" s="18" t="n"/>
-      <c r="G1" s="18" t="n"/>
-      <c r="H1" s="18" t="n"/>
-      <c r="I1" s="18" t="n"/>
-      <c r="J1" s="18" t="n"/>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
@@ -2306,10 +2314,6 @@
       <c r="D2" s="18" t="n"/>
       <c r="E2" s="18" t="n"/>
       <c r="F2" s="18" t="n"/>
-      <c r="G2" s="18" t="n"/>
-      <c r="H2" s="18" t="n"/>
-      <c r="I2" s="18" t="n"/>
-      <c r="J2" s="18" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="18" t="n"/>
@@ -2318,10 +2322,6 @@
       <c r="D3" s="18" t="n"/>
       <c r="E3" s="18" t="n"/>
       <c r="F3" s="18" t="n"/>
-      <c r="G3" s="18" t="n"/>
-      <c r="H3" s="18" t="n"/>
-      <c r="I3" s="18" t="n"/>
-      <c r="J3" s="18" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="18" t="n"/>
@@ -2331,25 +2331,21 @@
           <t>Event slot 1</t>
         </is>
       </c>
-      <c r="D4" s="18" t="n"/>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>Event slot 2</t>
+        </is>
+      </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>Event slot 2</t>
-        </is>
-      </c>
-      <c r="F4" s="18" t="n"/>
-      <c r="G4" s="21" t="inlineStr">
-        <is>
           <t>Event slot 3</t>
         </is>
       </c>
-      <c r="H4" s="18" t="n"/>
-      <c r="I4" s="21" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>Event slot 4</t>
         </is>
       </c>
-      <c r="J4" s="18" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
@@ -2369,7 +2365,7 @@
       </c>
       <c r="D5" s="20" t="inlineStr">
         <is>
-          <t>Test status</t>
+          <t>Expected value / rule</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -2379,27 +2375,7 @@
       </c>
       <c r="F5" s="20" t="inlineStr">
         <is>
-          <t>Test status</t>
-        </is>
-      </c>
-      <c r="G5" s="20" t="inlineStr">
-        <is>
           <t>Expected value / rule</t>
-        </is>
-      </c>
-      <c r="H5" s="20" t="inlineStr">
-        <is>
-          <t>Test status</t>
-        </is>
-      </c>
-      <c r="I5" s="20" t="inlineStr">
-        <is>
-          <t>Expected value / rule</t>
-        </is>
-      </c>
-      <c r="J5" s="20" t="inlineStr">
-        <is>
-          <t>Test status</t>
         </is>
       </c>
     </row>
@@ -2415,30 +2391,26 @@
           <t>page_view</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr"/>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
       <c r="E6" s="22" t="inlineStr">
         <is>
-          <t>search</t>
-        </is>
-      </c>
-      <c r="F6" s="22" t="inlineStr"/>
-      <c r="G6" s="22" t="inlineStr">
-        <is>
           <t>select_content</t>
         </is>
       </c>
-      <c r="H6" s="22" t="inlineStr"/>
-      <c r="I6" s="22" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>account_access_intent</t>
         </is>
       </c>
-      <c r="J6" s="22" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>event_classification</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
@@ -2448,49 +2420,29 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>EVT-HOME-PAGE-VIEW</t>
+          <t>automatic</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>recommended</t>
         </is>
       </c>
       <c r="E7" s="23" t="inlineStr">
         <is>
-          <t>EVT-HOME-SEARCH</t>
+          <t>recommended</t>
         </is>
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G7" s="23" t="inlineStr">
-        <is>
-          <t>EVT-HOME-CONTENT-SELECT</t>
-        </is>
-      </c>
-      <c r="H7" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I7" s="23" t="inlineStr">
-        <is>
-          <t>EVT-HOME-ACCOUNT-ACCESS</t>
-        </is>
-      </c>
-      <c r="J7" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>custom</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>event</t>
+          <t>trigger</t>
         </is>
       </c>
       <c r="B8" s="23" t="inlineStr">
@@ -2500,49 +2452,29 @@
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>page_view</t>
+          <t>Homepage load or SPA route change to the homepage.</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>User submits the site search form.</t>
         </is>
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>search</t>
+          <t>User clicks a consolidated navigation or content module.</t>
         </is>
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G8" s="23" t="inlineStr">
-        <is>
-          <t>select_content</t>
-        </is>
-      </c>
-      <c r="H8" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I8" s="23" t="inlineStr">
-        <is>
-          <t>account_access_intent</t>
-        </is>
-      </c>
-      <c r="J8" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>User clicks the account access entry point before the login result is known.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>event_classification</t>
+          <t>event</t>
         </is>
       </c>
       <c r="B9" s="23" t="inlineStr">
@@ -2552,101 +2484,61 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>automatic</t>
+          <t>page_view</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>search</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>recommended</t>
+          <t>select_content</t>
         </is>
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G9" s="23" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="H9" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I9" s="23" t="inlineStr">
-        <is>
-          <t>custom</t>
-        </is>
-      </c>
-      <c r="J9" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>account_access_intent</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>key_event</t>
+          <t>page_location</t>
         </is>
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>%current_url%</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G10" s="23" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H10" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I10" s="23" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="J10" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>page_or_component</t>
+          <t>page_title</t>
         </is>
       </c>
       <c r="B11" s="23" t="inlineStr">
@@ -2656,49 +2548,29 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Homepage document body</t>
+          <t>%document_title%</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E11" s="23" t="inlineStr">
         <is>
-          <t>Homepage search form</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G11" s="23" t="inlineStr">
-        <is>
-          <t>Homepage navigation, editorial, or service module</t>
-        </is>
-      </c>
-      <c r="H11" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I11" s="23" t="inlineStr">
-        <is>
-          <t>Homepage account access entry point</t>
-        </is>
-      </c>
-      <c r="J11" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>trigger</t>
+          <t>page_referrer</t>
         </is>
       </c>
       <c r="B12" s="23" t="inlineStr">
@@ -2708,49 +2580,29 @@
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Homepage load or SPA route change to the homepage.</t>
+          <t>%document_referrer%</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>User submits the site search form.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G12" s="23" t="inlineStr">
-        <is>
-          <t>User clicks a consolidated navigation or content module.</t>
-        </is>
-      </c>
-      <c r="H12" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I12" s="23" t="inlineStr">
-        <is>
-          <t>User clicks the account access entry point before the login result is known.</t>
-        </is>
-      </c>
-      <c r="J12" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t>screenshot_id</t>
+          <t>page_data.template</t>
         </is>
       </c>
       <c r="B13" s="23" t="inlineStr">
@@ -2760,49 +2612,29 @@
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>SCR-EVT-HOME-PAGE-VIEW</t>
+          <t>homepage</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E13" s="23" t="inlineStr">
         <is>
-          <t>SCR-EVT-HOME-SEARCH</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G13" s="23" t="inlineStr">
-        <is>
-          <t>SCR-EVT-HOME-CONTENT-SELECT</t>
-        </is>
-      </c>
-      <c r="H13" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I13" s="23" t="inlineStr">
-        <is>
-          <t>SCR-EVT-HOME-ACCOUNT-ACCESS</t>
-        </is>
-      </c>
-      <c r="J13" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t>qa_id</t>
+          <t>search_term</t>
         </is>
       </c>
       <c r="B14" s="23" t="inlineStr">
@@ -2812,49 +2644,29 @@
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>QA-HOME-PAGE-VIEW</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>%scrubbed_search_term%</t>
         </is>
       </c>
       <c r="E14" s="23" t="inlineStr">
         <is>
-          <t>QA-HOME-SEARCH</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G14" s="23" t="inlineStr">
-        <is>
-          <t>QA-HOME-CONTENT-SELECT</t>
-        </is>
-      </c>
-      <c r="H14" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I14" s="23" t="inlineStr">
-        <is>
-          <t>QA-HOME-ACCOUNT-ACCESS</t>
-        </is>
-      </c>
-      <c r="J14" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>page_location</t>
+          <t>content_type</t>
         </is>
       </c>
       <c r="B15" s="23" t="inlineStr">
@@ -2864,49 +2676,29 @@
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>%current_url%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E15" s="23" t="inlineStr">
         <is>
+          <t>category_navigation | editorial_module | service_link</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G15" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H15" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I15" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J15" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
         <is>
-          <t>page_title</t>
+          <t>content_id</t>
         </is>
       </c>
       <c r="B16" s="23" t="inlineStr">
@@ -2916,49 +2708,29 @@
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>%document_title%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
+          <t>%stable_content_id%</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G16" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H16" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I16" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J16" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>page_referrer</t>
+          <t>content_name</t>
         </is>
       </c>
       <c r="B17" s="23" t="inlineStr">
@@ -2968,49 +2740,29 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>%document_referrer%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
         <is>
+          <t>%normalized_content_name%</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J17" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>page_data.template</t>
+          <t>cta_location</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
@@ -3020,49 +2772,29 @@
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>homepage</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E18" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>header | hero | body | footer</t>
         </is>
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G18" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I18" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J18" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>header | menu</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>search_term</t>
+          <t>link_url</t>
         </is>
       </c>
       <c r="B19" s="23" t="inlineStr">
@@ -3077,44 +2809,24 @@
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E19" s="23" t="inlineStr">
         <is>
-          <t>%scrubbed_search_term%</t>
+          <t>%destination_url%</t>
         </is>
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G19" s="23" t="inlineStr">
-        <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I19" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>content_type</t>
+          <t>cta_text</t>
         </is>
       </c>
       <c r="B20" s="23" t="inlineStr">
@@ -3129,7 +2841,7 @@
       </c>
       <c r="D20" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E20" s="23" t="inlineStr">
@@ -3139,34 +2851,14 @@
       </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G20" s="23" t="inlineStr">
-        <is>
-          <t>category_navigation | editorial_module | service_link</t>
-        </is>
-      </c>
-      <c r="H20" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I20" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
+          <t>%normalized_cta_text%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>content_id</t>
+          <t>login_status</t>
         </is>
       </c>
       <c r="B21" s="23" t="inlineStr">
@@ -3181,7 +2873,7 @@
       </c>
       <c r="D21" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E21" s="23" t="inlineStr">
@@ -3191,86 +2883,34 @@
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G21" s="23" t="inlineStr">
-        <is>
-          <t>%stable_content_id%</t>
-        </is>
-      </c>
-      <c r="H21" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I21" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J21" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="23" t="inlineStr">
-        <is>
-          <t>content_name</t>
-        </is>
-      </c>
-      <c r="B22" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C22" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D22" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E22" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F22" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G22" s="23" t="inlineStr">
-        <is>
-          <t>%normalized_content_name%</t>
-        </is>
-      </c>
-      <c r="H22" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I22" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
+          <t>logged | not_logged | unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>J-002 - Homepage discovery - Ecommerce promotions</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr"/>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>view_promotion</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>select_promotion</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr"/>
+      <c r="F22" s="22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
         <is>
-          <t>cta_location</t>
+          <t>event_classification</t>
         </is>
       </c>
       <c r="B23" s="23" t="inlineStr">
@@ -3280,49 +2920,21 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>recommended_ecommerce</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E23" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G23" s="23" t="inlineStr">
-        <is>
-          <t>header | hero | body | footer</t>
-        </is>
-      </c>
-      <c r="H23" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I23" s="23" t="inlineStr">
-        <is>
-          <t>header | menu</t>
-        </is>
-      </c>
-      <c r="J23" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
+          <t>recommended_ecommerce</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="inlineStr"/>
+      <c r="F23" s="23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
         <is>
-          <t>link_url</t>
+          <t>trigger</t>
         </is>
       </c>
       <c r="B24" s="23" t="inlineStr">
@@ -3332,49 +2944,21 @@
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promotion module is visible according to the agreed impression threshold.</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E24" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G24" s="23" t="inlineStr">
-        <is>
-          <t>%destination_url%</t>
-        </is>
-      </c>
-      <c r="H24" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I24" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
+          <t>User clicks a tracked homepage promotion.</t>
+        </is>
+      </c>
+      <c r="E24" s="23" t="inlineStr"/>
+      <c r="F24" s="23" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>cta_text</t>
+          <t>event</t>
         </is>
       </c>
       <c r="B25" s="23" t="inlineStr">
@@ -3384,49 +2968,21 @@
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>view_promotion</t>
         </is>
       </c>
       <c r="D25" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E25" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G25" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I25" s="23" t="inlineStr">
-        <is>
-          <t>%normalized_cta_text%</t>
-        </is>
-      </c>
-      <c r="J25" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
+          <t>select_promotion</t>
+        </is>
+      </c>
+      <c r="E25" s="23" t="inlineStr"/>
+      <c r="F25" s="23" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>login_status</t>
+          <t>currency</t>
         </is>
       </c>
       <c r="B26" s="23" t="inlineStr">
@@ -3434,75 +2990,47 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C26" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D26" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E26" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G26" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H26" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I26" s="23" t="inlineStr">
-        <is>
-          <t>logged | not_logged | unknown</t>
-        </is>
-      </c>
-      <c r="J26" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="22" t="inlineStr">
-        <is>
-          <t>J-002 - Homepage discovery - Ecommerce promotions</t>
-        </is>
-      </c>
-      <c r="B27" s="22" t="inlineStr"/>
-      <c r="C27" s="22" t="inlineStr">
-        <is>
-          <t>view_promotion</t>
-        </is>
-      </c>
-      <c r="D27" s="22" t="inlineStr"/>
-      <c r="E27" s="22" t="inlineStr">
-        <is>
-          <t>select_promotion</t>
-        </is>
-      </c>
-      <c r="F27" s="22" t="inlineStr"/>
-      <c r="G27" s="22" t="inlineStr"/>
-      <c r="H27" s="22" t="inlineStr"/>
-      <c r="I27" s="22" t="inlineStr"/>
-      <c r="J27" s="22" t="inlineStr"/>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E26" s="23" t="inlineStr"/>
+      <c r="F26" s="23" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>promotion_id</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="inlineStr">
+        <is>
+          <t>%promotion_id%</t>
+        </is>
+      </c>
+      <c r="D27" s="23" t="inlineStr">
+        <is>
+          <t>%promotion_id%</t>
+        </is>
+      </c>
+      <c r="E27" s="23" t="inlineStr"/>
+      <c r="F27" s="23" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>promotion_name</t>
         </is>
       </c>
       <c r="B28" s="23" t="inlineStr">
@@ -3512,33 +3040,21 @@
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
-          <t>EVT-HOME-PROMO-VIEW</t>
+          <t>%promotion_name%</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E28" s="23" t="inlineStr">
-        <is>
-          <t>EVT-HOME-PROMO-SELECT</t>
-        </is>
-      </c>
-      <c r="F28" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G28" s="23" t="inlineStr"/>
-      <c r="H28" s="23" t="inlineStr"/>
-      <c r="I28" s="23" t="inlineStr"/>
-      <c r="J28" s="23" t="inlineStr"/>
+          <t>%promotion_name%</t>
+        </is>
+      </c>
+      <c r="E28" s="23" t="inlineStr"/>
+      <c r="F28" s="23" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="23" t="inlineStr">
         <is>
-          <t>event</t>
+          <t>creative_name</t>
         </is>
       </c>
       <c r="B29" s="23" t="inlineStr">
@@ -3548,33 +3064,21 @@
       </c>
       <c r="C29" s="23" t="inlineStr">
         <is>
-          <t>view_promotion</t>
+          <t>%creative_name%</t>
         </is>
       </c>
       <c r="D29" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E29" s="23" t="inlineStr">
-        <is>
-          <t>select_promotion</t>
-        </is>
-      </c>
-      <c r="F29" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G29" s="23" t="inlineStr"/>
-      <c r="H29" s="23" t="inlineStr"/>
-      <c r="I29" s="23" t="inlineStr"/>
-      <c r="J29" s="23" t="inlineStr"/>
+          <t>%creative_name%</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr"/>
+      <c r="F29" s="23" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
-          <t>event_classification</t>
+          <t>creative_slot</t>
         </is>
       </c>
       <c r="B30" s="23" t="inlineStr">
@@ -3584,69 +3088,45 @@
       </c>
       <c r="C30" s="23" t="inlineStr">
         <is>
-          <t>recommended_ecommerce</t>
+          <t>%creative_slot%</t>
         </is>
       </c>
       <c r="D30" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>recommended_ecommerce</t>
-        </is>
-      </c>
-      <c r="F30" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G30" s="23" t="inlineStr"/>
-      <c r="H30" s="23" t="inlineStr"/>
-      <c r="I30" s="23" t="inlineStr"/>
-      <c r="J30" s="23" t="inlineStr"/>
+          <t>%creative_slot%</t>
+        </is>
+      </c>
+      <c r="E30" s="23" t="inlineStr"/>
+      <c r="F30" s="23" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="23" t="inlineStr">
         <is>
-          <t>key_event</t>
+          <t>items</t>
         </is>
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>array&lt;object&gt;</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>Array&lt;Item&gt;; see items[] rows below</t>
         </is>
       </c>
       <c r="D31" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E31" s="23" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F31" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G31" s="23" t="inlineStr"/>
-      <c r="H31" s="23" t="inlineStr"/>
-      <c r="I31" s="23" t="inlineStr"/>
-      <c r="J31" s="23" t="inlineStr"/>
+          <t>Array&lt;Item&gt;; see items[] rows below</t>
+        </is>
+      </c>
+      <c r="E31" s="23" t="inlineStr"/>
+      <c r="F31" s="23" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="23" t="inlineStr">
         <is>
-          <t>page_or_component</t>
+          <t>items[].item_id</t>
         </is>
       </c>
       <c r="B32" s="23" t="inlineStr">
@@ -3656,33 +3136,21 @@
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>Homepage merchandising promotion module</t>
+          <t>%promotion_item_id%</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E32" s="23" t="inlineStr">
-        <is>
-          <t>Homepage merchandising promotion link or card</t>
-        </is>
-      </c>
-      <c r="F32" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G32" s="23" t="inlineStr"/>
-      <c r="H32" s="23" t="inlineStr"/>
-      <c r="I32" s="23" t="inlineStr"/>
-      <c r="J32" s="23" t="inlineStr"/>
+          <t>%promotion_item_id%</t>
+        </is>
+      </c>
+      <c r="E32" s="23" t="inlineStr"/>
+      <c r="F32" s="23" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="23" t="inlineStr">
         <is>
-          <t>trigger</t>
+          <t>items[].item_name</t>
         </is>
       </c>
       <c r="B33" s="23" t="inlineStr">
@@ -3692,33 +3160,21 @@
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>Promotion module is visible according to the agreed impression threshold.</t>
+          <t>%promotion_item_name%</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
         <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E33" s="23" t="inlineStr">
-        <is>
-          <t>User clicks a tracked homepage promotion.</t>
-        </is>
-      </c>
-      <c r="F33" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G33" s="23" t="inlineStr"/>
-      <c r="H33" s="23" t="inlineStr"/>
-      <c r="I33" s="23" t="inlineStr"/>
-      <c r="J33" s="23" t="inlineStr"/>
+          <t>%promotion_item_name%</t>
+        </is>
+      </c>
+      <c r="E33" s="23" t="inlineStr"/>
+      <c r="F33" s="23" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
         <is>
-          <t>screenshot_id</t>
+          <t>items[].affiliation</t>
         </is>
       </c>
       <c r="B34" s="23" t="inlineStr">
@@ -3726,35 +3182,23 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C34" s="23" t="inlineStr">
-        <is>
-          <t>SCR-EVT-HOME-PROMO-VIEW</t>
-        </is>
-      </c>
-      <c r="D34" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E34" s="23" t="inlineStr">
-        <is>
-          <t>SCR-EVT-HOME-PROMO-SELECT</t>
-        </is>
-      </c>
-      <c r="F34" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G34" s="23" t="inlineStr"/>
-      <c r="H34" s="23" t="inlineStr"/>
-      <c r="I34" s="23" t="inlineStr"/>
-      <c r="J34" s="23" t="inlineStr"/>
+      <c r="C34" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D34" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E34" s="23" t="inlineStr"/>
+      <c r="F34" s="23" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>qa_id</t>
+          <t>items[].coupon</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
@@ -3762,40 +3206,28 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C35" s="23" t="inlineStr">
-        <is>
-          <t>QA-HOME-PROMO-VIEW</t>
-        </is>
-      </c>
-      <c r="D35" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E35" s="23" t="inlineStr">
-        <is>
-          <t>QA-HOME-PROMO-SELECT</t>
-        </is>
-      </c>
-      <c r="F35" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G35" s="23" t="inlineStr"/>
-      <c r="H35" s="23" t="inlineStr"/>
-      <c r="I35" s="23" t="inlineStr"/>
-      <c r="J35" s="23" t="inlineStr"/>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E35" s="23" t="inlineStr"/>
+      <c r="F35" s="23" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>items[].discount</t>
         </is>
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="C36" s="24" t="inlineStr">
@@ -3803,66 +3235,42 @@
           <t>not_available</t>
         </is>
       </c>
-      <c r="D36" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E36" s="24" t="inlineStr">
+      <c r="D36" s="24" t="inlineStr">
         <is>
           <t>not_available</t>
         </is>
       </c>
-      <c r="F36" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G36" s="23" t="inlineStr"/>
-      <c r="H36" s="23" t="inlineStr"/>
-      <c r="I36" s="23" t="inlineStr"/>
-      <c r="J36" s="23" t="inlineStr"/>
+      <c r="E36" s="23" t="inlineStr"/>
+      <c r="F36" s="23" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>promotion_id</t>
+          <t>items[].index</t>
         </is>
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C37" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_id%</t>
-        </is>
-      </c>
-      <c r="D37" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E37" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_id%</t>
-        </is>
-      </c>
-      <c r="F37" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G37" s="23" t="inlineStr"/>
-      <c r="H37" s="23" t="inlineStr"/>
-      <c r="I37" s="23" t="inlineStr"/>
-      <c r="J37" s="23" t="inlineStr"/>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="C37" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E37" s="23" t="inlineStr"/>
+      <c r="F37" s="23" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="23" t="inlineStr">
         <is>
-          <t>promotion_name</t>
+          <t>items[].item_brand</t>
         </is>
       </c>
       <c r="B38" s="23" t="inlineStr">
@@ -3870,35 +3278,23 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C38" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_name%</t>
-        </is>
-      </c>
-      <c r="D38" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E38" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_name%</t>
-        </is>
-      </c>
-      <c r="F38" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G38" s="23" t="inlineStr"/>
-      <c r="H38" s="23" t="inlineStr"/>
-      <c r="I38" s="23" t="inlineStr"/>
-      <c r="J38" s="23" t="inlineStr"/>
+      <c r="C38" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D38" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="inlineStr"/>
+      <c r="F38" s="23" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
         <is>
-          <t>creative_name</t>
+          <t>items[].item_category</t>
         </is>
       </c>
       <c r="B39" s="23" t="inlineStr">
@@ -3906,35 +3302,23 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C39" s="23" t="inlineStr">
-        <is>
-          <t>%creative_name%</t>
-        </is>
-      </c>
-      <c r="D39" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E39" s="23" t="inlineStr">
-        <is>
-          <t>%creative_name%</t>
-        </is>
-      </c>
-      <c r="F39" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G39" s="23" t="inlineStr"/>
-      <c r="H39" s="23" t="inlineStr"/>
-      <c r="I39" s="23" t="inlineStr"/>
-      <c r="J39" s="23" t="inlineStr"/>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E39" s="23" t="inlineStr"/>
+      <c r="F39" s="23" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="23" t="inlineStr">
         <is>
-          <t>creative_slot</t>
+          <t>items[].item_category2</t>
         </is>
       </c>
       <c r="B40" s="23" t="inlineStr">
@@ -3942,71 +3326,47 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C40" s="23" t="inlineStr">
-        <is>
-          <t>%creative_slot%</t>
-        </is>
-      </c>
-      <c r="D40" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E40" s="23" t="inlineStr">
-        <is>
-          <t>%creative_slot%</t>
-        </is>
-      </c>
-      <c r="F40" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G40" s="23" t="inlineStr"/>
-      <c r="H40" s="23" t="inlineStr"/>
-      <c r="I40" s="23" t="inlineStr"/>
-      <c r="J40" s="23" t="inlineStr"/>
+      <c r="C40" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E40" s="23" t="inlineStr"/>
+      <c r="F40" s="23" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>items[].item_category3</t>
         </is>
       </c>
       <c r="B41" s="23" t="inlineStr">
         <is>
-          <t>array&lt;object&gt;</t>
-        </is>
-      </c>
-      <c r="C41" s="23" t="inlineStr">
-        <is>
-          <t>Array&lt;Item&gt;; see items[] rows below</t>
-        </is>
-      </c>
-      <c r="D41" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E41" s="23" t="inlineStr">
-        <is>
-          <t>Array&lt;Item&gt;; see items[] rows below</t>
-        </is>
-      </c>
-      <c r="F41" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G41" s="23" t="inlineStr"/>
-      <c r="H41" s="23" t="inlineStr"/>
-      <c r="I41" s="23" t="inlineStr"/>
-      <c r="J41" s="23" t="inlineStr"/>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C41" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D41" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="inlineStr"/>
+      <c r="F41" s="23" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
         <is>
-          <t>items[].item_id</t>
+          <t>items[].item_category4</t>
         </is>
       </c>
       <c r="B42" s="23" t="inlineStr">
@@ -4014,35 +3374,23 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C42" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_item_id%</t>
-        </is>
-      </c>
-      <c r="D42" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E42" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_item_id%</t>
-        </is>
-      </c>
-      <c r="F42" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G42" s="23" t="inlineStr"/>
-      <c r="H42" s="23" t="inlineStr"/>
-      <c r="I42" s="23" t="inlineStr"/>
-      <c r="J42" s="23" t="inlineStr"/>
+      <c r="C42" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D42" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E42" s="23" t="inlineStr"/>
+      <c r="F42" s="23" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>items[].item_name</t>
+          <t>items[].item_category5</t>
         </is>
       </c>
       <c r="B43" s="23" t="inlineStr">
@@ -4050,35 +3398,23 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C43" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_item_name%</t>
-        </is>
-      </c>
-      <c r="D43" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E43" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_item_name%</t>
-        </is>
-      </c>
-      <c r="F43" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G43" s="23" t="inlineStr"/>
-      <c r="H43" s="23" t="inlineStr"/>
-      <c r="I43" s="23" t="inlineStr"/>
-      <c r="J43" s="23" t="inlineStr"/>
+      <c r="C43" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D43" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="E43" s="23" t="inlineStr"/>
+      <c r="F43" s="23" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t>items[].affiliation</t>
+          <t>items[].item_list_id</t>
         </is>
       </c>
       <c r="B44" s="23" t="inlineStr">
@@ -4091,30 +3427,18 @@
           <t>not_available</t>
         </is>
       </c>
-      <c r="D44" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E44" s="24" t="inlineStr">
+      <c r="D44" s="24" t="inlineStr">
         <is>
           <t>not_available</t>
         </is>
       </c>
-      <c r="F44" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G44" s="23" t="inlineStr"/>
-      <c r="H44" s="23" t="inlineStr"/>
-      <c r="I44" s="23" t="inlineStr"/>
-      <c r="J44" s="23" t="inlineStr"/>
+      <c r="E44" s="23" t="inlineStr"/>
+      <c r="F44" s="23" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>items[].coupon</t>
+          <t>items[].item_list_name</t>
         </is>
       </c>
       <c r="B45" s="23" t="inlineStr">
@@ -4127,35 +3451,23 @@
           <t>not_available</t>
         </is>
       </c>
-      <c r="D45" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E45" s="24" t="inlineStr">
+      <c r="D45" s="24" t="inlineStr">
         <is>
           <t>not_available</t>
         </is>
       </c>
-      <c r="F45" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G45" s="23" t="inlineStr"/>
-      <c r="H45" s="23" t="inlineStr"/>
-      <c r="I45" s="23" t="inlineStr"/>
-      <c r="J45" s="23" t="inlineStr"/>
+      <c r="E45" s="23" t="inlineStr"/>
+      <c r="F45" s="23" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t>items[].discount</t>
+          <t>items[].item_variant</t>
         </is>
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C46" s="24" t="inlineStr">
@@ -4163,35 +3475,23 @@
           <t>not_available</t>
         </is>
       </c>
-      <c r="D46" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E46" s="24" t="inlineStr">
+      <c r="D46" s="24" t="inlineStr">
         <is>
           <t>not_available</t>
         </is>
       </c>
-      <c r="F46" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G46" s="23" t="inlineStr"/>
-      <c r="H46" s="23" t="inlineStr"/>
-      <c r="I46" s="23" t="inlineStr"/>
-      <c r="J46" s="23" t="inlineStr"/>
+      <c r="E46" s="23" t="inlineStr"/>
+      <c r="F46" s="23" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="23" t="inlineStr">
         <is>
-          <t>items[].index</t>
+          <t>items[].location_id</t>
         </is>
       </c>
       <c r="B47" s="23" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C47" s="24" t="inlineStr">
@@ -4199,35 +3499,23 @@
           <t>not_available</t>
         </is>
       </c>
-      <c r="D47" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E47" s="24" t="inlineStr">
+      <c r="D47" s="24" t="inlineStr">
         <is>
           <t>not_available</t>
         </is>
       </c>
-      <c r="F47" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G47" s="23" t="inlineStr"/>
-      <c r="H47" s="23" t="inlineStr"/>
-      <c r="I47" s="23" t="inlineStr"/>
-      <c r="J47" s="23" t="inlineStr"/>
+      <c r="E47" s="23" t="inlineStr"/>
+      <c r="F47" s="23" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="23" t="inlineStr">
         <is>
-          <t>items[].item_brand</t>
+          <t>items[].price</t>
         </is>
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="C48" s="24" t="inlineStr">
@@ -4235,66 +3523,42 @@
           <t>not_available</t>
         </is>
       </c>
-      <c r="D48" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E48" s="24" t="inlineStr">
+      <c r="D48" s="24" t="inlineStr">
         <is>
           <t>not_available</t>
         </is>
       </c>
-      <c r="F48" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G48" s="23" t="inlineStr"/>
-      <c r="H48" s="23" t="inlineStr"/>
-      <c r="I48" s="23" t="inlineStr"/>
-      <c r="J48" s="23" t="inlineStr"/>
+      <c r="E48" s="23" t="inlineStr"/>
+      <c r="F48" s="23" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category</t>
+          <t>items[].quantity</t>
         </is>
       </c>
       <c r="B49" s="23" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C49" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D49" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E49" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F49" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G49" s="23" t="inlineStr"/>
-      <c r="H49" s="23" t="inlineStr"/>
-      <c r="I49" s="23" t="inlineStr"/>
-      <c r="J49" s="23" t="inlineStr"/>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="C49" s="25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" s="25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E49" s="23" t="inlineStr"/>
+      <c r="F49" s="23" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category2</t>
+          <t>items[].creative_name</t>
         </is>
       </c>
       <c r="B50" s="23" t="inlineStr">
@@ -4302,35 +3566,23 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C50" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D50" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E50" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F50" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G50" s="23" t="inlineStr"/>
-      <c r="H50" s="23" t="inlineStr"/>
-      <c r="I50" s="23" t="inlineStr"/>
-      <c r="J50" s="23" t="inlineStr"/>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>event-level creative_name: %creative_name%</t>
+        </is>
+      </c>
+      <c r="D50" s="26" t="inlineStr">
+        <is>
+          <t>event-level creative_name: %creative_name%</t>
+        </is>
+      </c>
+      <c r="E50" s="23" t="inlineStr"/>
+      <c r="F50" s="23" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category3</t>
+          <t>items[].creative_slot</t>
         </is>
       </c>
       <c r="B51" s="23" t="inlineStr">
@@ -4338,35 +3590,23 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C51" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D51" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E51" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F51" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G51" s="23" t="inlineStr"/>
-      <c r="H51" s="23" t="inlineStr"/>
-      <c r="I51" s="23" t="inlineStr"/>
-      <c r="J51" s="23" t="inlineStr"/>
+      <c r="C51" s="26" t="inlineStr">
+        <is>
+          <t>event-level creative_slot: %creative_slot%</t>
+        </is>
+      </c>
+      <c r="D51" s="26" t="inlineStr">
+        <is>
+          <t>event-level creative_slot: %creative_slot%</t>
+        </is>
+      </c>
+      <c r="E51" s="23" t="inlineStr"/>
+      <c r="F51" s="23" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category4</t>
+          <t>items[].promotion_id</t>
         </is>
       </c>
       <c r="B52" s="23" t="inlineStr">
@@ -4374,35 +3614,23 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C52" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D52" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E52" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F52" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G52" s="23" t="inlineStr"/>
-      <c r="H52" s="23" t="inlineStr"/>
-      <c r="I52" s="23" t="inlineStr"/>
-      <c r="J52" s="23" t="inlineStr"/>
+      <c r="C52" s="26" t="inlineStr">
+        <is>
+          <t>event-level promotion_id: %promotion_id%</t>
+        </is>
+      </c>
+      <c r="D52" s="26" t="inlineStr">
+        <is>
+          <t>event-level promotion_id: %promotion_id%</t>
+        </is>
+      </c>
+      <c r="E52" s="23" t="inlineStr"/>
+      <c r="F52" s="23" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category5</t>
+          <t>items[].promotion_name</t>
         </is>
       </c>
       <c r="B53" s="23" t="inlineStr">
@@ -4410,450 +3638,25 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C53" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D53" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E53" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F53" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G53" s="23" t="inlineStr"/>
-      <c r="H53" s="23" t="inlineStr"/>
-      <c r="I53" s="23" t="inlineStr"/>
-      <c r="J53" s="23" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="23" t="inlineStr">
-        <is>
-          <t>items[].item_list_id</t>
-        </is>
-      </c>
-      <c r="B54" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C54" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D54" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E54" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F54" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G54" s="23" t="inlineStr"/>
-      <c r="H54" s="23" t="inlineStr"/>
-      <c r="I54" s="23" t="inlineStr"/>
-      <c r="J54" s="23" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="23" t="inlineStr">
-        <is>
-          <t>items[].item_list_name</t>
-        </is>
-      </c>
-      <c r="B55" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C55" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D55" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E55" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F55" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G55" s="23" t="inlineStr"/>
-      <c r="H55" s="23" t="inlineStr"/>
-      <c r="I55" s="23" t="inlineStr"/>
-      <c r="J55" s="23" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="23" t="inlineStr">
-        <is>
-          <t>items[].item_variant</t>
-        </is>
-      </c>
-      <c r="B56" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C56" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D56" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E56" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F56" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G56" s="23" t="inlineStr"/>
-      <c r="H56" s="23" t="inlineStr"/>
-      <c r="I56" s="23" t="inlineStr"/>
-      <c r="J56" s="23" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="23" t="inlineStr">
-        <is>
-          <t>items[].location_id</t>
-        </is>
-      </c>
-      <c r="B57" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C57" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D57" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E57" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F57" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G57" s="23" t="inlineStr"/>
-      <c r="H57" s="23" t="inlineStr"/>
-      <c r="I57" s="23" t="inlineStr"/>
-      <c r="J57" s="23" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="23" t="inlineStr">
-        <is>
-          <t>items[].price</t>
-        </is>
-      </c>
-      <c r="B58" s="23" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="C58" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D58" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E58" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="F58" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G58" s="23" t="inlineStr"/>
-      <c r="H58" s="23" t="inlineStr"/>
-      <c r="I58" s="23" t="inlineStr"/>
-      <c r="J58" s="23" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="23" t="inlineStr">
-        <is>
-          <t>items[].quantity</t>
-        </is>
-      </c>
-      <c r="B59" s="23" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="C59" s="25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D59" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E59" s="25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F59" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G59" s="23" t="inlineStr"/>
-      <c r="H59" s="23" t="inlineStr"/>
-      <c r="I59" s="23" t="inlineStr"/>
-      <c r="J59" s="23" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="23" t="inlineStr">
-        <is>
-          <t>items[].creative_name</t>
-        </is>
-      </c>
-      <c r="B60" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C60" s="26" t="inlineStr">
-        <is>
-          <t>event-level creative_name: %creative_name%</t>
-        </is>
-      </c>
-      <c r="D60" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E60" s="26" t="inlineStr">
-        <is>
-          <t>event-level creative_name: %creative_name%</t>
-        </is>
-      </c>
-      <c r="F60" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G60" s="23" t="inlineStr"/>
-      <c r="H60" s="23" t="inlineStr"/>
-      <c r="I60" s="23" t="inlineStr"/>
-      <c r="J60" s="23" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="23" t="inlineStr">
-        <is>
-          <t>items[].creative_slot</t>
-        </is>
-      </c>
-      <c r="B61" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C61" s="26" t="inlineStr">
-        <is>
-          <t>event-level creative_slot: %creative_slot%</t>
-        </is>
-      </c>
-      <c r="D61" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E61" s="26" t="inlineStr">
-        <is>
-          <t>event-level creative_slot: %creative_slot%</t>
-        </is>
-      </c>
-      <c r="F61" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G61" s="23" t="inlineStr"/>
-      <c r="H61" s="23" t="inlineStr"/>
-      <c r="I61" s="23" t="inlineStr"/>
-      <c r="J61" s="23" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="23" t="inlineStr">
-        <is>
-          <t>items[].promotion_id</t>
-        </is>
-      </c>
-      <c r="B62" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C62" s="26" t="inlineStr">
-        <is>
-          <t>event-level promotion_id: %promotion_id%</t>
-        </is>
-      </c>
-      <c r="D62" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E62" s="26" t="inlineStr">
-        <is>
-          <t>event-level promotion_id: %promotion_id%</t>
-        </is>
-      </c>
-      <c r="F62" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G62" s="23" t="inlineStr"/>
-      <c r="H62" s="23" t="inlineStr"/>
-      <c r="I62" s="23" t="inlineStr"/>
-      <c r="J62" s="23" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="23" t="inlineStr">
-        <is>
-          <t>items[].promotion_name</t>
-        </is>
-      </c>
-      <c r="B63" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C63" s="26" t="inlineStr">
+      <c r="C53" s="26" t="inlineStr">
         <is>
           <t>event-level promotion_name: %promotion_name%</t>
         </is>
       </c>
-      <c r="D63" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="E63" s="26" t="inlineStr">
+      <c r="D53" s="26" t="inlineStr">
         <is>
           <t>event-level promotion_name: %promotion_name%</t>
         </is>
       </c>
-      <c r="F63" s="23" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="G63" s="23" t="inlineStr"/>
-      <c r="H63" s="23" t="inlineStr"/>
-      <c r="I63" s="23" t="inlineStr"/>
-      <c r="J63" s="23" t="inlineStr"/>
+      <c r="E53" s="23" t="inlineStr"/>
+      <c r="F53" s="23" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:J63"/>
-  <mergeCells count="6">
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="C4:D4"/>
+  <autoFilter ref="A5:F53"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D6:D2000">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"KO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
-      <formula>"Cannot test"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F6:F2000">
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
-      <formula>"KO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2">
-      <formula>"Cannot test"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H6:H2000">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="1">
-      <formula>"KO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="2">
-      <formula>"Cannot test"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J6:J2000">
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="1">
-      <formula>"KO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="2">
-      <formula>"Cannot test"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="D6:D2000 F6:F2000 H6:H2000 J6:J2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"OK,KO,Cannot test"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4869,13 +3672,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -4895,7 +3698,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Attach or link screenshots used to validate Event Matrix rows.</t>
+          <t>Capture requirements and visual evidence for later recette.</t>
         </is>
       </c>
       <c r="B2" s="18" t="n"/>
@@ -4909,37 +3712,37 @@
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>Screenshot ID</t>
+          <t>Journey</t>
         </is>
       </c>
       <c r="B3" s="20" t="inlineStr">
         <is>
-          <t>Journey</t>
+          <t>Event</t>
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>Event name</t>
+          <t>Page / component</t>
         </is>
       </c>
       <c r="D3" s="20" t="inlineStr">
         <is>
-          <t>Page / component</t>
+          <t>URL / route</t>
         </is>
       </c>
       <c r="E3" s="20" t="inlineStr">
         <is>
-          <t>URL / route</t>
+          <t>Capture objective</t>
         </is>
       </c>
       <c r="F3" s="20" t="inlineStr">
         <is>
-          <t>What to capture</t>
+          <t>Automation cue</t>
         </is>
       </c>
       <c r="G3" s="20" t="inlineStr">
         <is>
-          <t>File path or link</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="H3" s="20" t="inlineStr">
@@ -4951,228 +3754,252 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
         <is>
-          <t>SCR-EVT-HOME-PAGE-VIEW</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>page_view</t>
         </is>
       </c>
       <c r="C4" s="18" t="inlineStr">
         <is>
-          <t>page_view</t>
+          <t>Homepage document body</t>
         </is>
       </c>
       <c r="D4" s="18" t="inlineStr">
         <is>
-          <t>Homepage document body</t>
+          <t>https://example.com/</t>
         </is>
       </c>
       <c r="E4" s="18" t="inlineStr">
         <is>
-          <t>https://example.com/</t>
+          <t>Homepage document body - Homepage load or SPA route change to the homepage.</t>
         </is>
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Homepage document body - Homepage load or SPA route change to the homepage.</t>
-        </is>
-      </c>
-      <c r="G4" s="18" t="inlineStr"/>
+          <t>Open the route and capture the rendered page state.</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>capture_required</t>
+        </is>
+      </c>
       <c r="H4" s="18" t="inlineStr">
         <is>
-          <t>QA case: QA-HOME-PAGE-VIEW</t>
+          <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="56" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>SCR-EVT-HOME-PROMO-VIEW</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>view_promotion</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>view_promotion</t>
+          <t>Homepage merchandising promotion module</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>Homepage merchandising promotion module</t>
+          <t>https://example.com/</t>
         </is>
       </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>https://example.com/</t>
+          <t>Homepage merchandising promotion module - Promotion module is visible according to the agreed impression threshold.</t>
         </is>
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>Homepage merchandising promotion module - Promotion module is visible according to the agreed impression threshold.</t>
-        </is>
-      </c>
-      <c r="G5" s="18" t="inlineStr"/>
+          <t>Open the route and reproduce the ecommerce state before validating GA4 payload.</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>capture_required</t>
+        </is>
+      </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
-          <t>QA case: QA-HOME-PROMO-VIEW</t>
+          <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="56" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>SCR-EVT-HOME-PROMO-SELECT</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>select_promotion</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>select_promotion</t>
+          <t>Homepage merchandising promotion link or card</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>Homepage merchandising promotion link or card</t>
+          <t>https://example.com/</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>https://example.com/</t>
+          <t>Homepage merchandising promotion link or card - User clicks a tracked homepage promotion.</t>
         </is>
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>Homepage merchandising promotion link or card - User clicks a tracked homepage promotion.</t>
-        </is>
-      </c>
-      <c r="G6" s="18" t="inlineStr"/>
+          <t>Open the route and reproduce the ecommerce state before validating GA4 payload.</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>capture_required</t>
+        </is>
+      </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>QA case: QA-HOME-PROMO-SELECT</t>
+          <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="56" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>SCR-EVT-HOME-SEARCH</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>search</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>search</t>
+          <t>Homepage search form</t>
         </is>
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Homepage search form</t>
+          <t>https://example.com/</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>https://example.com/</t>
+          <t>Homepage search form - User submits the site search form.</t>
         </is>
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>Homepage search form - User submits the site search form.</t>
-        </is>
-      </c>
-      <c r="G7" s="18" t="inlineStr"/>
+          <t>Open the route and capture the rendered page state.</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>capture_required</t>
+        </is>
+      </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>QA case: QA-HOME-SEARCH</t>
+          <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="56" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>SCR-EVT-HOME-CONTENT-SELECT</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>select_content</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>select_content</t>
+          <t>Homepage navigation, editorial, or service module</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>Homepage navigation, editorial, or service module</t>
+          <t>https://example.com/</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>https://example.com/</t>
+          <t>Homepage navigation, editorial, or service module - User clicks a consolidated navigation or content module.</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Homepage navigation, editorial, or service module - User clicks a consolidated navigation or content module.</t>
-        </is>
-      </c>
-      <c r="G8" s="18" t="inlineStr"/>
+          <t>Open the route and capture the rendered page state.</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>capture_required</t>
+        </is>
+      </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>QA case: QA-HOME-CONTENT-SELECT</t>
+          <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="56" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>SCR-EVT-HOME-ACCOUNT-ACCESS</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>account_access_intent</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>account_access_intent</t>
+          <t>Homepage account access entry point</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Homepage account access entry point</t>
+          <t>https://example.com/</t>
         </is>
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>https://example.com/</t>
+          <t>Homepage account access entry point - User clicks the account access entry point before the login result is known.</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Homepage account access entry point - User clicks the account access entry point before the login result is known.</t>
-        </is>
-      </c>
-      <c r="G9" s="18" t="inlineStr"/>
+          <t>Open the route and capture the rendered page state.</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>capture_required</t>
+        </is>
+      </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>QA case: QA-HOME-ACCOUNT-ACCESS</t>
+          <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
@@ -5182,6 +4009,28 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <conditionalFormatting sqref="G4:G209">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"captured"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"shared_evidence"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"capture_required"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"blocked"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+      <formula>"not_needed"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="G4:G209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"capture_required,captured,shared_evidence,not_needed,blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5240,17 +4089,17 @@
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>QA ID</t>
+          <t>Event name</t>
         </is>
       </c>
       <c r="B3" s="20" t="inlineStr">
         <is>
-          <t>Event name</t>
+          <t>Journey</t>
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>Journey</t>
+          <t>Page / component</t>
         </is>
       </c>
       <c r="D3" s="20" t="inlineStr">
@@ -5287,17 +4136,17 @@
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
         <is>
-          <t>QA-HOME-PAGE-VIEW</t>
+          <t>page_view</t>
         </is>
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>page_view</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="C4" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>Homepage document body</t>
         </is>
       </c>
       <c r="D4" s="18" t="inlineStr">
@@ -5336,17 +4185,17 @@
     <row r="5">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>QA-HOME-PROMO-VIEW</t>
+          <t>view_promotion</t>
         </is>
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>view_promotion</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>Homepage merchandising promotion module</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
@@ -5385,17 +4234,17 @@
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>QA-HOME-PROMO-SELECT</t>
+          <t>select_promotion</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>select_promotion</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>Homepage merchandising promotion link or card</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
@@ -5433,17 +4282,17 @@
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>QA-HOME-SEARCH</t>
+          <t>search</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>search</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>Homepage search form</t>
         </is>
       </c>
       <c r="D7" s="18" t="inlineStr">
@@ -5481,17 +4330,17 @@
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t>QA-HOME-CONTENT-SELECT</t>
+          <t>select_content</t>
         </is>
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>select_content</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>Homepage navigation, editorial, or service module</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
@@ -5530,17 +4379,17 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>QA-HOME-ACCOUNT-ACCESS</t>
+          <t>account_access_intent</t>
         </is>
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>account_access_intent</t>
+          <t>Homepage discovery</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>Homepage discovery</t>
+          <t>Homepage account access entry point</t>
         </is>
       </c>
       <c r="D9" s="18" t="inlineStr">
@@ -5586,7 +4435,7 @@
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="3">
       <formula>"KO"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">

</xml_diff>

<commit_message>
Improve GA4 tracking plan release package
</commit_message>
<xml_diff>
--- a/skill/assets/ga4_tracking_plan_template.xlsx
+++ b/skill/assets/ga4_tracking_plan_template.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 GTM Protocol'!$A$3:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Parameter Reference'!$A$3:$I$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Event Matrix'!$A$5:$F$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Screenshot Register'!$A$3:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Screenshot Register'!$A$3:$I$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05 QA Cases'!$A$3:$I$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3675,17 +3675,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3701,6 +3702,7 @@
       <c r="F1" s="18" t="n"/>
       <c r="G1" s="18" t="n"/>
       <c r="H1" s="18" t="n"/>
+      <c r="I1" s="18" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
@@ -3715,6 +3717,7 @@
       <c r="F2" s="18" t="n"/>
       <c r="G2" s="18" t="n"/>
       <c r="H2" s="18" t="n"/>
+      <c r="I2" s="18" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
@@ -3729,36 +3732,41 @@
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
+          <t>Screenshot preview</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
           <t>Page / component</t>
         </is>
       </c>
-      <c r="D3" s="20" t="inlineStr">
+      <c r="E3" s="20" t="inlineStr">
         <is>
           <t>URL / route</t>
         </is>
       </c>
-      <c r="E3" s="20" t="inlineStr">
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>Capture objective</t>
         </is>
       </c>
-      <c r="F3" s="20" t="inlineStr">
+      <c r="G3" s="20" t="inlineStr">
         <is>
           <t>Automation cue</t>
         </is>
       </c>
-      <c r="G3" s="20" t="inlineStr">
+      <c r="H3" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H3" s="20" t="inlineStr">
+      <c r="I3" s="20" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="56" customHeight="1">
+    <row r="4" ht="132" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -3769,38 +3777,39 @@
           <t>page_view</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr"/>
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Homepage document body</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>https://example.com/</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Homepage document body - Homepage load or SPA route change to the homepage.</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Open the route and capture the rendered page state.</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>capture_required</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="56" customHeight="1">
+    <row r="5" ht="132" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -3811,38 +3820,39 @@
           <t>view_promotion</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr"/>
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>Homepage merchandising promotion module</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
         <is>
           <t>https://example.com/</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="F5" s="18" t="inlineStr">
         <is>
           <t>Homepage merchandising promotion module - Promotion module is visible according to the agreed impression threshold.</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="G5" s="18" t="inlineStr">
         <is>
           <t>Open the route and reproduce the ecommerce state before validating GA4 payload.</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>capture_required</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1">
+    <row r="6" ht="132" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -3853,38 +3863,39 @@
           <t>select_promotion</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr"/>
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>Homepage merchandising promotion link or card</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>https://example.com/</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>Homepage merchandising promotion link or card - User clicks a tracked homepage promotion.</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="G6" s="18" t="inlineStr">
         <is>
           <t>Open the route and reproduce the ecommerce state before validating GA4 payload.</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>capture_required</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="I6" s="18" t="inlineStr">
         <is>
           <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="56" customHeight="1">
+    <row r="7" ht="132" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -3895,38 +3906,39 @@
           <t>search</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr"/>
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>Homepage search form</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>https://example.com/</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>Homepage search form - User submits the site search form.</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="G7" s="18" t="inlineStr">
         <is>
           <t>Open the route and capture the rendered page state.</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="H7" s="18" t="inlineStr">
         <is>
           <t>capture_required</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="I7" s="18" t="inlineStr">
         <is>
           <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="56" customHeight="1">
+    <row r="8" ht="132" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -3937,38 +3949,39 @@
           <t>select_content</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr"/>
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Homepage navigation, editorial, or service module</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>https://example.com/</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="F8" s="18" t="inlineStr">
         <is>
           <t>Homepage navigation, editorial, or service module - User clicks a consolidated navigation or content module.</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="G8" s="18" t="inlineStr">
         <is>
           <t>Open the route and capture the rendered page state.</t>
         </is>
       </c>
-      <c r="G8" s="18" t="inlineStr">
+      <c r="H8" s="18" t="inlineStr">
         <is>
           <t>capture_required</t>
         </is>
       </c>
-      <c r="H8" s="18" t="inlineStr">
+      <c r="I8" s="18" t="inlineStr">
         <is>
           <t>Capture during coverage or later QA when the journey is accessible.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="56" customHeight="1">
+    <row r="9" ht="132" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -3979,44 +3992,45 @@
           <t>account_access_intent</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr"/>
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>Homepage account access entry point</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>https://example.com/</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
         <is>
           <t>Homepage account access entry point - User clicks the account access entry point before the login result is known.</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="G9" s="18" t="inlineStr">
         <is>
           <t>Skip or capture only with approved test access; do not use personal credentials.</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="H9" s="18" t="inlineStr">
         <is>
           <t>skip_allowed</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="I9" s="18" t="inlineStr">
         <is>
           <t>Skip is allowed when approved credentials or a safe test environment are unavailable.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H9"/>
+  <autoFilter ref="A3:I9"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G4:G209">
+  <conditionalFormatting sqref="H4:H209">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"captured"</formula>
     </cfRule>
@@ -4037,7 +4051,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G4:G209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H4:H209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"capture_required,captured,shared_evidence,skip_allowed,not_needed,blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Release GA4-only tracking plan skill v1
</commit_message>
<xml_diff>
--- a/skill/assets/ga4_tracking_plan_template.xlsx
+++ b/skill/assets/ga4_tracking_plan_template.xlsx
@@ -12,14 +12,12 @@
     <sheet name="02 Parameter Reference" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="03 Event Matrix" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="04 Screenshot Register" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05 QA Cases" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 GTM Protocol'!$A$3:$D$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Parameter Reference'!$A$3:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 GTM Protocol'!$A$3:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Parameter Reference'!$A$3:$K$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Event Matrix'!$A$5:$F$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Screenshot Register'!$A$3:$I$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05 QA Cases'!$A$3:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Screenshot Register'!$A$3:$H$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -723,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -801,7 +799,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Last update</t>
+          <t>Publish date</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -823,16 +821,8 @@
           <t>v0.1</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>GA4</t>
-        </is>
-      </c>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr"/>
       <c r="E5" s="7" t="inlineStr"/>
       <c r="F5" s="8" t="inlineStr"/>
       <c r="G5" s="7" t="inlineStr"/>
@@ -985,7 +975,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Capture requirements and visual evidence for later recette.</t>
+          <t>Page and interaction evidence supporting implementation.</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr"/>
@@ -995,116 +985,94 @@
       <c r="H13" s="13" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>05 QA Cases</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>Manual recette checks and validation status.</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr"/>
-      <c r="E14" s="16" t="inlineStr"/>
-      <c r="F14" s="16" t="inlineStr"/>
-      <c r="G14" s="16" t="inlineStr"/>
-      <c r="H14" s="16" t="inlineStr"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="9" t="inlineStr"/>
-      <c r="B15" s="9" t="inlineStr"/>
-      <c r="C15" s="9" t="inlineStr"/>
-      <c r="D15" s="9" t="inlineStr"/>
-      <c r="E15" s="9" t="inlineStr"/>
-      <c r="F15" s="9" t="inlineStr"/>
-      <c r="G15" s="9" t="inlineStr"/>
-      <c r="H15" s="9" t="inlineStr"/>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr"/>
+      <c r="B14" s="9" t="inlineStr"/>
+      <c r="C14" s="9" t="inlineStr"/>
+      <c r="D14" s="9" t="inlineStr"/>
+      <c r="E14" s="9" t="inlineStr"/>
+      <c r="F14" s="9" t="inlineStr"/>
+      <c r="G14" s="9" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Version History</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="4" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>Publish date</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr"/>
-      <c r="G17" s="10" t="inlineStr"/>
-      <c r="H17" s="10" t="inlineStr"/>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr"/>
+      <c r="G16" s="10" t="inlineStr"/>
+      <c r="H16" s="10" t="inlineStr"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>v0.1</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>Tracking plan draft generated for review.</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr"/>
-      <c r="G18" s="16" t="inlineStr"/>
-      <c r="H18" s="16" t="inlineStr"/>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>GA4 tracking plan prepared for review.</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr"/>
+      <c r="G17" s="13" t="inlineStr"/>
+      <c r="H17" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A15:H15"/>
     <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -1114,7 +1082,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -1127,7 +1094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1297,37 +1264,15 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>QA status</t>
+          <t>Official references</t>
         </is>
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>Record execution status in QA Cases or Screenshot Register, not inside the Event Matrix.</t>
+          <t>Check current official documentation before approving standard, recommended, ecommerce, and GTM dataLayer decisions.</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>OK / KO / Cannot test / captured</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Keep the Event Matrix focused on implementation rules.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Official references</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Check current official documentation before approving standard, recommended, ecommerce, and GTM dataLayer decisions.</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>GA4 recommended events: https://developers.google.com/analytics/devguides/collection/ga4/reference/events
 GA4 ecommerce: https://developers.google.com/analytics/devguides/collection/ga4/ecommerce
@@ -1335,14 +1280,14 @@
 GTM dataLayer: https://developers.google.com/tag-platform/tag-manager/datalayer</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>Keep external references here, not on the Overview tab.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D10"/>
+  <autoFilter ref="A3:D9"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -1358,18 +1303,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1386,6 +1333,8 @@
       <c r="G1" s="18" t="n"/>
       <c r="H1" s="18" t="n"/>
       <c r="I1" s="18" t="n"/>
+      <c r="J1" s="18" t="n"/>
+      <c r="K1" s="18" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
@@ -1401,6 +1350,8 @@
       <c r="G2" s="18" t="n"/>
       <c r="H2" s="18" t="n"/>
       <c r="I2" s="18" t="n"/>
+      <c r="J2" s="18" t="n"/>
+      <c r="K2" s="18" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
@@ -1440,10 +1391,20 @@
       </c>
       <c r="H3" s="20" t="inlineStr">
         <is>
+          <t>Availability</t>
+        </is>
+      </c>
+      <c r="I3" s="20" t="inlineStr">
+        <is>
+          <t>Data owner</t>
+        </is>
+      </c>
+      <c r="J3" s="20" t="inlineStr">
+        <is>
           <t>Register in GA4</t>
         </is>
       </c>
-      <c r="I3" s="20" t="inlineStr">
+      <c r="K3" s="20" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
@@ -1485,8 +1446,22 @@
           <t>https://example.com/</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr"/>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium; PII risk: medium</t>
         </is>
@@ -1528,8 +1503,22 @@
           <t>Homepage</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr"/>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J5" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K5" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium</t>
         </is>
@@ -1571,8 +1560,22 @@
           <t>https://www.google.com/</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr"/>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J6" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium; PII risk: medium</t>
         </is>
@@ -1614,8 +1617,22 @@
           <t>homepage</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr"/>
-      <c r="I7" s="18" t="inlineStr"/>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J7" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K7" s="18" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
@@ -1653,8 +1670,22 @@
           <t>home_hero_summer_2026</t>
         </is>
       </c>
-      <c r="H8" s="18" t="inlineStr"/>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J8" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium</t>
         </is>
@@ -1696,8 +1727,22 @@
           <t>summer_sale</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr"/>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J9" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K9" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium</t>
         </is>
@@ -1739,8 +1784,22 @@
           <t>banner_blue</t>
         </is>
       </c>
-      <c r="H10" s="18" t="inlineStr"/>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I10" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J10" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K10" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium</t>
         </is>
@@ -1782,8 +1841,22 @@
           <t>homepage_hero_1</t>
         </is>
       </c>
-      <c r="H11" s="18" t="inlineStr"/>
-      <c r="I11" s="18" t="inlineStr"/>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J11" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K11" s="18" t="inlineStr"/>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
@@ -1821,8 +1894,22 @@
           <t>[{item_id:'sku_123',item_name:'summer_dress'}]</t>
         </is>
       </c>
-      <c r="H12" s="18" t="inlineStr"/>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I12" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J12" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K12" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium</t>
         </is>
@@ -1864,8 +1951,22 @@
           <t>sku_123</t>
         </is>
       </c>
-      <c r="H13" s="18" t="inlineStr"/>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I13" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J13" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K13" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: high</t>
         </is>
@@ -1907,8 +2008,22 @@
           <t>summer_dress</t>
         </is>
       </c>
-      <c r="H14" s="18" t="inlineStr"/>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I14" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J14" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K14" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: high</t>
         </is>
@@ -1950,8 +2065,22 @@
           <t>summer_dress</t>
         </is>
       </c>
-      <c r="H15" s="18" t="inlineStr"/>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I15" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J15" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K15" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: high; PII risk: medium</t>
         </is>
@@ -1995,10 +2124,20 @@
       </c>
       <c r="H16" s="18" t="inlineStr">
         <is>
-          <t>Yes - custom_dimension (should)</t>
-        </is>
-      </c>
-      <c r="I16" s="18" t="inlineStr"/>
+          <t>to_confirm</t>
+        </is>
+      </c>
+      <c r="I16" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K16" s="18" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="18" t="inlineStr">
@@ -2038,10 +2177,20 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>Yes - custom_dimension (should)</t>
+          <t>to_confirm</t>
         </is>
       </c>
       <c r="I17" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J17" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K17" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium</t>
         </is>
@@ -2085,10 +2234,20 @@
       </c>
       <c r="H18" s="18" t="inlineStr">
         <is>
-          <t>Yes - custom_dimension (could)</t>
+          <t>to_confirm</t>
         </is>
       </c>
       <c r="I18" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J18" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K18" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium</t>
         </is>
@@ -2132,10 +2291,20 @@
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>Yes - custom_dimension (should)</t>
-        </is>
-      </c>
-      <c r="I19" s="18" t="inlineStr"/>
+          <t>to_confirm</t>
+        </is>
+      </c>
+      <c r="I19" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J19" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K19" s="18" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
@@ -2173,8 +2342,22 @@
           <t>https://example.com/category/women</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr"/>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
       <c r="I20" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J20" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K20" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: high; PII risk: medium</t>
         </is>
@@ -2218,10 +2401,20 @@
       </c>
       <c r="H21" s="18" t="inlineStr">
         <is>
-          <t>Yes - custom_dimension (could)</t>
+          <t>to_confirm</t>
         </is>
       </c>
       <c r="I21" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J21" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K21" s="18" t="inlineStr">
         <is>
           <t>Cardinality risk: medium</t>
         </is>
@@ -2265,16 +2458,26 @@
       </c>
       <c r="H22" s="18" t="inlineStr">
         <is>
-          <t>Yes - custom_dimension (could)</t>
-        </is>
-      </c>
-      <c r="I22" s="18" t="inlineStr"/>
+          <t>to_confirm</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>Web analyst and development team</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K22" s="18" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:I22"/>
+  <autoFilter ref="A3:K22"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -3675,18 +3878,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3702,12 +3904,11 @@
       <c r="F1" s="18" t="n"/>
       <c r="G1" s="18" t="n"/>
       <c r="H1" s="18" t="n"/>
-      <c r="I1" s="18" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Capture requirements and visual evidence for later recette.</t>
+          <t>Page and interaction evidence supporting the Event Matrix.</t>
         </is>
       </c>
       <c r="B2" s="18" t="n"/>
@@ -3717,7 +3918,6 @@
       <c r="F2" s="18" t="n"/>
       <c r="G2" s="18" t="n"/>
       <c r="H2" s="18" t="n"/>
-      <c r="I2" s="18" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
@@ -3727,7 +3927,7 @@
       </c>
       <c r="B3" s="20" t="inlineStr">
         <is>
-          <t>Event</t>
+          <t>Event(s)</t>
         </is>
       </c>
       <c r="C3" s="20" t="inlineStr">
@@ -3752,15 +3952,10 @@
       </c>
       <c r="G3" s="20" t="inlineStr">
         <is>
-          <t>Automation cue</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3790,22 +3985,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Homepage document body - Homepage load or SPA route change to the homepage.</t>
+          <t>Show Homepage document body for page_view.</t>
         </is>
       </c>
       <c r="G4" s="18" t="inlineStr">
         <is>
-          <t>Open the route and capture the rendered page state.</t>
+          <t>capture_required</t>
         </is>
       </c>
       <c r="H4" s="18" t="inlineStr">
         <is>
-          <t>capture_required</t>
-        </is>
-      </c>
-      <c r="I4" s="18" t="inlineStr">
-        <is>
-          <t>Capture during coverage or later QA when the journey is accessible.</t>
+          <t>Capture a representative page state or clearly identify the tracked interaction.</t>
         </is>
       </c>
     </row>
@@ -3833,22 +4023,17 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>Homepage merchandising promotion module - Promotion module is visible according to the agreed impression threshold.</t>
+          <t>Show Homepage merchandising promotion module for view_promotion.</t>
         </is>
       </c>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>Open the route and reproduce the ecommerce state before validating GA4 payload.</t>
+          <t>capture_required</t>
         </is>
       </c>
       <c r="H5" s="18" t="inlineStr">
         <is>
-          <t>capture_required</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>Capture during coverage or later QA when the journey is accessible.</t>
+          <t>Capture a representative page state or clearly identify the tracked interaction.</t>
         </is>
       </c>
     </row>
@@ -3876,22 +4061,17 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>Homepage merchandising promotion link or card - User clicks a tracked homepage promotion.</t>
+          <t>Show Homepage merchandising promotion link or card for select_promotion.</t>
         </is>
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Open the route and reproduce the ecommerce state before validating GA4 payload.</t>
+          <t>capture_required</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>capture_required</t>
-        </is>
-      </c>
-      <c r="I6" s="18" t="inlineStr">
-        <is>
-          <t>Capture during coverage or later QA when the journey is accessible.</t>
+          <t>Capture a representative page state or clearly identify the tracked interaction.</t>
         </is>
       </c>
     </row>
@@ -3919,22 +4099,17 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>Homepage search form - User submits the site search form.</t>
+          <t>Show Homepage search form for search.</t>
         </is>
       </c>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>Open the route and capture the rendered page state.</t>
+          <t>capture_required</t>
         </is>
       </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>capture_required</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>Capture during coverage or later QA when the journey is accessible.</t>
+          <t>Capture a representative page state or clearly identify the tracked interaction.</t>
         </is>
       </c>
     </row>
@@ -3962,22 +4137,17 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Homepage navigation, editorial, or service module - User clicks a consolidated navigation or content module.</t>
+          <t>Show Homepage navigation, editorial, or service module for select_content.</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
         <is>
-          <t>Open the route and capture the rendered page state.</t>
+          <t>capture_required</t>
         </is>
       </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>capture_required</t>
-        </is>
-      </c>
-      <c r="I8" s="18" t="inlineStr">
-        <is>
-          <t>Capture during coverage or later QA when the journey is accessible.</t>
+          <t>Capture a representative page state or clearly identify the tracked interaction.</t>
         </is>
       </c>
     </row>
@@ -4005,32 +4175,27 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Homepage account access entry point - User clicks the account access entry point before the login result is known.</t>
+          <t>Show Homepage account access entry point for account_access_intent.</t>
         </is>
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>Skip or capture only with approved test access; do not use personal credentials.</t>
+          <t>skip_allowed</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>skip_allowed</t>
-        </is>
-      </c>
-      <c r="I9" s="18" t="inlineStr">
-        <is>
           <t>Skip is allowed when approved credentials or a safe test environment are unavailable.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:I9"/>
+  <autoFilter ref="A3:H9"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H4:H209">
+  <conditionalFormatting sqref="G4:G209">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"captured"</formula>
     </cfRule>
@@ -4051,427 +4216,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G4:G209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"capture_required,captured,shared_evidence,skip_allowed,not_needed,blocked"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:I9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="54" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
-    <col width="56" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>QA Cases</t>
-        </is>
-      </c>
-      <c r="B1" s="18" t="n"/>
-      <c r="C1" s="18" t="n"/>
-      <c r="D1" s="18" t="n"/>
-      <c r="E1" s="18" t="n"/>
-      <c r="F1" s="18" t="n"/>
-      <c r="G1" s="18" t="n"/>
-      <c r="H1" s="18" t="n"/>
-      <c r="I1" s="18" t="n"/>
-    </row>
-    <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="19" t="inlineStr">
-        <is>
-          <t>Manual recette checklist for the events in the Event Matrix.</t>
-        </is>
-      </c>
-      <c r="B2" s="18" t="n"/>
-      <c r="C2" s="18" t="n"/>
-      <c r="D2" s="18" t="n"/>
-      <c r="E2" s="18" t="n"/>
-      <c r="F2" s="18" t="n"/>
-      <c r="G2" s="18" t="n"/>
-      <c r="H2" s="18" t="n"/>
-      <c r="I2" s="18" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Event name</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>Journey</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>Page / component</t>
-        </is>
-      </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>Test method</t>
-        </is>
-      </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>Test steps</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Expected dataLayer</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Expected GA4 / network</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
-        <is>
-          <t>Evidence / notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t>page_view</t>
-        </is>
-      </c>
-      <c r="B4" s="18" t="inlineStr">
-        <is>
-          <t>Homepage discovery</t>
-        </is>
-      </c>
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>Homepage document body</t>
-        </is>
-      </c>
-      <c r="D4" s="18" t="inlineStr">
-        <is>
-          <t>DebugView | GTM Preview | Network</t>
-        </is>
-      </c>
-      <c r="E4" s="18" t="inlineStr">
-        <is>
-          <t>Open https://example.com/ once.</t>
-        </is>
-      </c>
-      <c r="F4" s="18" t="inlineStr">
-        <is>
-          <t>page_data.location equals current URL.
-page_data.template equals homepage.</t>
-        </is>
-      </c>
-      <c r="G4" s="18" t="inlineStr">
-        <is>
-          <t>en=page_view
-page_location populated</t>
-        </is>
-      </c>
-      <c r="H4" s="18" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I4" s="18" t="inlineStr">
-        <is>
-          <t>One homepage page_view appears.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>view_promotion</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Homepage discovery</t>
-        </is>
-      </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>Homepage merchandising promotion module</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>GTM Preview | Network</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Expose a tracked promotion.</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>ecommerce object is flushed.
-promotion_id and items are present.</t>
-        </is>
-      </c>
-      <c r="G5" s="18" t="inlineStr">
-        <is>
-          <t>en=view_promotion
-promotion_id and item identifier present</t>
-        </is>
-      </c>
-      <c r="H5" s="18" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>view_promotion appears for the qualified impression.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>select_promotion</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Homepage discovery</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>Homepage merchandising promotion link or card</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>GTM Preview | Network</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>Click a tracked promotion.</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>select_promotion uses the same promotion_id as view_promotion.</t>
-        </is>
-      </c>
-      <c r="G6" s="18" t="inlineStr">
-        <is>
-          <t>en=select_promotion
-promotion_id and item identifier present</t>
-        </is>
-      </c>
-      <c r="H6" s="18" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I6" s="18" t="inlineStr">
-        <is>
-          <t>select_promotion appears after click.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>search</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Homepage discovery</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>Homepage search form</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>DebugView | GTM Preview | Network</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>Submit a safe search query.</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>event_data.search_term is present and scrubbed.</t>
-        </is>
-      </c>
-      <c r="G7" s="18" t="inlineStr">
-        <is>
-          <t>en=search
-search_term populated</t>
-        </is>
-      </c>
-      <c r="H7" s="18" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>search appears with search_term.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>select_content</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Homepage discovery</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>Homepage navigation, editorial, or service module</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>GTM Preview | Network</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Click one representative content or navigation module.</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>event_data.content_type uses an allowed value.
-content_id identifies the selected module.</t>
-        </is>
-      </c>
-      <c r="G8" s="18" t="inlineStr">
-        <is>
-          <t>en=select_content
-content_type and content_id present</t>
-        </is>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I8" s="18" t="inlineStr">
-        <is>
-          <t>select_content appears with controlled values.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>account_access_intent</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Homepage discovery</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>Homepage account access entry point</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>GTM Preview | Network</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Click the account access entry point.</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>event_data.cta_location is present.
-user_data.login_status is logged, not_logged, or unknown.</t>
-        </is>
-      </c>
-      <c r="G9" s="18" t="inlineStr">
-        <is>
-          <t>en=account_access_intent
-No direct personal identifiers are present</t>
-        </is>
-      </c>
-      <c r="H9" s="18" t="inlineStr">
-        <is>
-          <t>Cannot test</t>
-        </is>
-      </c>
-      <c r="I9" s="18" t="inlineStr">
-        <is>
-          <t>account_access_intent appears on account entry click.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:I9"/>
-  <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-  </mergeCells>
-  <conditionalFormatting sqref="H4:H209">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
-      <formula>"KO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
-      <formula>"Cannot test"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="H4:H209" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"OK,KO,Cannot test"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup fitToHeight="0" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Harden GA4 tracking plans for connected users
</commit_message>
<xml_diff>
--- a/skill/assets/ga4_tracking_plan_template.xlsx
+++ b/skill/assets/ga4_tracking_plan_template.xlsx
@@ -11,13 +11,15 @@
     <sheet name="01 GTM Protocol" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="02 Parameter Reference" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="03 Event Matrix" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04 Screenshot Register" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="04 DataLayer Examples" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05 Screenshot Register" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 GTM Protocol'!$A$3:$D$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Parameter Reference'!$A$3:$K$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Event Matrix'!$A$5:$F$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 Screenshot Register'!$A$3:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 GTM Protocol'!$A$3:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 Parameter Reference'!$A$3:$K$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03 Event Matrix'!$A$5:$F$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04 DataLayer Examples'!$A$3:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05 Screenshot Register'!$A$3:$H$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -721,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -970,12 +972,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>04 Screenshot Register</t>
+          <t>04 DataLayer Examples</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Page and interaction evidence supporting implementation.</t>
+          <t>Complete per-event GTM and dataLayer implementation examples.</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr"/>
@@ -985,94 +987,116 @@
       <c r="H13" s="13" t="inlineStr"/>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="9" t="inlineStr"/>
-      <c r="B14" s="9" t="inlineStr"/>
-      <c r="C14" s="9" t="inlineStr"/>
-      <c r="D14" s="9" t="inlineStr"/>
-      <c r="E14" s="9" t="inlineStr"/>
-      <c r="F14" s="9" t="inlineStr"/>
-      <c r="G14" s="9" t="inlineStr"/>
-      <c r="H14" s="9" t="inlineStr"/>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>05 Screenshot Register</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>Page and interaction evidence supporting implementation.</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr"/>
+      <c r="E14" s="16" t="inlineStr"/>
+      <c r="F14" s="16" t="inlineStr"/>
+      <c r="G14" s="16" t="inlineStr"/>
+      <c r="H14" s="16" t="inlineStr"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="9" t="inlineStr"/>
+      <c r="B15" s="9" t="inlineStr"/>
+      <c r="C15" s="9" t="inlineStr"/>
+      <c r="D15" s="9" t="inlineStr"/>
+      <c r="E15" s="9" t="inlineStr"/>
+      <c r="F15" s="9" t="inlineStr"/>
+      <c r="G15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr"/>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Version History</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
-      <c r="H15" s="4" t="n"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>Publish date</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr"/>
-      <c r="G16" s="10" t="inlineStr"/>
-      <c r="H16" s="10" t="inlineStr"/>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="F17" s="10" t="inlineStr"/>
+      <c r="G17" s="10" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>v0.1</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>GA4 tracking plan prepared for review.</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="F17" s="13" t="inlineStr"/>
-      <c r="G17" s="13" t="inlineStr"/>
-      <c r="H17" s="13" t="inlineStr"/>
+      <c r="F18" s="16" t="inlineStr"/>
+      <c r="G18" s="16" t="inlineStr"/>
+      <c r="H18" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A15:H15"/>
     <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -1082,6 +1106,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
@@ -1094,7 +1119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1264,30 +1289,155 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
+          <t>Consent</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Set and update consent through the CMP or GTM consent APIs before affected tags process user or event data.</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>analytics_storage
+ad_storage
+ad_user_data
+ad_personalization</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>The tracking plan records dependencies but does not make the legal consent decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Connected user context</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Push user_context independently when authentication state is known, after successful login, and after logout. Do not repeat these fields inside every event push.</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>dataLayer.push({
+  user_context: {
+    user_id: "%opaque_user_id%",
+    login_status: "logged_in",
+    customer_status: "returning",
+    account_type: "standard"
+  }
+});</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Plan status: planned. Keep the object available before dependent GA4 events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>GA4 User-ID</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Map user_context.user_id only to the Google tag user_id setting. Omit before first sign-in and set null after logout.</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>user_context.user_id -&gt; Google tag user_id</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Never send user_id as an event parameter or user property, and never register it as a custom dimension.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>GA4 user properties</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Map only approved low-cardinality connected-user fields as GA4 user properties.</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>user_context.login_status -&gt; GA4 user property login_status
+user_context.customer_status -&gt; GA4 user property customer_status
+user_context.account_type -&gt; GA4 user property account_type</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Register planned custom user properties in GA4. Do not include direct identifiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Advertising user data</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Keep direct identifiers in a separately governed non-GA4 object only when another approved advertising implementation explicitly requires them.</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Direct identifiers are not sent to GA4. Define them only in a separate advertising implementation when explicitly required and approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
           <t>Official references</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Check current official documentation before approving standard, recommended, ecommerce, and GTM dataLayer decisions.</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Check current official documentation before approving standard, recommended, ecommerce, connected-user, and GTM dataLayer decisions.</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>GA4 recommended events: https://developers.google.com/analytics/devguides/collection/ga4/reference/events
 GA4 ecommerce: https://developers.google.com/analytics/devguides/collection/ga4/ecommerce
 GA4 item parameters: https://developers.google.com/analytics/devguides/collection/ga4/item-scoped-ecommerce
-GTM dataLayer: https://developers.google.com/tag-platform/tag-manager/datalayer</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
+GA4 User-ID: https://developers.google.com/analytics/devguides/collection/ga4/user-id
+GA4 user properties: https://developers.google.com/analytics/devguides/collection/protocol/ga4/user-properties
+GTM dataLayer: https://developers.google.com/tag-platform/tag-manager/datalayer
+Consent mode: https://developers.google.com/tag-platform/security/guides/consent</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
         <is>
           <t>Keep external references here, not on the Overview tab.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D9"/>
+  <autoFilter ref="A3:D14"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -1303,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1406,7 +1556,7 @@
       </c>
       <c r="K3" s="20" t="inlineStr">
         <is>
-          <t>Comments</t>
+          <t>Privacy / consent</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1613,7 @@
       </c>
       <c r="K4" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium; PII risk: medium</t>
+          <t>Cardinality risk: medium; PII risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1670,7 @@
       </c>
       <c r="K5" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium</t>
+          <t>Cardinality risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1727,7 @@
       </c>
       <c r="K6" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium; PII risk: medium</t>
+          <t>Cardinality risk: medium; PII risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1759,7 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>Use controlled lowercase ASCII snake_case values.</t>
+          <t>homepage | listing_page | product_page | cart | checkout | content_page</t>
         </is>
       </c>
       <c r="G7" s="18" t="inlineStr">
@@ -1687,7 +1837,7 @@
       </c>
       <c r="K8" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium</t>
+          <t>Cardinality risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1894,7 @@
       </c>
       <c r="K9" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium</t>
+          <t>Cardinality risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1951,7 @@
       </c>
       <c r="K10" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium</t>
+          <t>Cardinality risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -1856,7 +2006,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="K11" s="18" t="inlineStr"/>
+      <c r="K11" s="18" t="inlineStr">
+        <is>
+          <t>Consent: analytics_storage</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
@@ -1911,7 +2065,7 @@
       </c>
       <c r="K12" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium</t>
+          <t>Cardinality risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -1968,7 +2122,7 @@
       </c>
       <c r="K13" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: high</t>
+          <t>Cardinality risk: high; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2179,7 @@
       </c>
       <c r="K14" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: high</t>
+          <t>Cardinality risk: high; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2236,7 @@
       </c>
       <c r="K15" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: high; PII risk: medium</t>
+          <t>Cardinality risk: high; PII risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2268,7 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>Use controlled lowercase ASCII snake_case values.</t>
+          <t>category_navigation | editorial_module | service_link</t>
         </is>
       </c>
       <c r="G16" s="18" t="inlineStr">
@@ -2137,7 +2291,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K16" s="18" t="inlineStr"/>
+      <c r="K16" s="18" t="inlineStr">
+        <is>
+          <t>Consent: analytics_storage</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="18" t="inlineStr">
@@ -2192,7 +2350,7 @@
       </c>
       <c r="K17" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium</t>
+          <t>Cardinality risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2407,7 @@
       </c>
       <c r="K18" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium</t>
+          <t>Cardinality risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2439,7 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Use controlled lowercase ASCII snake_case values.</t>
+          <t>header | hero | body | footer | menu</t>
         </is>
       </c>
       <c r="G19" s="18" t="inlineStr">
@@ -2304,7 +2462,11 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K19" s="18" t="inlineStr"/>
+      <c r="K19" s="18" t="inlineStr">
+        <is>
+          <t>Consent: analytics_storage</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
@@ -2359,7 +2521,7 @@
       </c>
       <c r="K20" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: high; PII risk: medium</t>
+          <t>Cardinality risk: high; PII risk: medium; Consent: analytics_storage</t>
         </is>
       </c>
     </row>
@@ -2416,65 +2578,240 @@
       </c>
       <c r="K21" s="18" t="inlineStr">
         <is>
-          <t>Cardinality risk: medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
+          <t>Cardinality risk: medium; Consent: analytics_storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
       <c r="A22" s="18" t="inlineStr">
         <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>GA4 User ID</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>implementation</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Opaque stable authenticated identifier mapped only to the GA4 User-ID configuration setting.</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>Use a stable non-PII internal identifier. Omit before sign-in and set null after logout. Never use email or register this value as a custom dimension.</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>usr_7f3a91</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>requires_development</t>
+        </is>
+      </c>
+      <c r="I22" s="18" t="inlineStr">
+        <is>
+          <t>Authentication and analytics teams</t>
+        </is>
+      </c>
+      <c r="J22" s="18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K22" s="18" t="inlineStr">
+        <is>
+          <t>Cardinality risk: high; PII risk: medium; Consent: analytics_storage and organization-approved User-ID policy; Implementation-only: do not map to ordinary GA4 parameters</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
           <t>login_status</t>
         </is>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>Login status</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>event</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
         <is>
           <t>Known anonymous login state.</t>
         </is>
       </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>Use logged | not_logged | unknown.</t>
-        </is>
-      </c>
-      <c r="G22" s="18" t="inlineStr">
-        <is>
-          <t>not_logged</t>
-        </is>
-      </c>
-      <c r="H22" s="18" t="inlineStr">
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>logged_in | logged_out</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>logged_out</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
         <is>
           <t>to_confirm</t>
         </is>
       </c>
-      <c r="I22" s="18" t="inlineStr">
+      <c r="I23" s="18" t="inlineStr">
         <is>
           <t>Web analyst and development team</t>
         </is>
       </c>
-      <c r="J22" s="18" t="inlineStr">
+      <c r="J23" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K22" s="18" t="inlineStr"/>
+      <c r="K23" s="18" t="inlineStr">
+        <is>
+          <t>Consent: analytics_storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>customer_status</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Customer status</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Low-cardinality customer lifecycle group available after authentication.</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>new | returning | unknown</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>returning</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>CRM and analytics teams</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K24" s="18" t="inlineStr">
+        <is>
+          <t>Consent: analytics_storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>account_type</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Account type</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Optional low-cardinality account category when the business has stable account types.</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>Use a small English controlled taxonomy defined by the business; omit when no meaningful account categories exist.</t>
+        </is>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>to_confirm</t>
+        </is>
+      </c>
+      <c r="I25" s="18" t="inlineStr">
+        <is>
+          <t>CRM and analytics teams</t>
+        </is>
+      </c>
+      <c r="J25" s="18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K25" s="18" t="inlineStr">
+        <is>
+          <t>Consent: analytics_storage</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K22"/>
+  <autoFilter ref="A3:K25"/>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
@@ -2490,7 +2827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2592,7 +2929,7 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t>J-001 - Homepage discovery - Interactions</t>
+          <t>J-001 - Homepage discovery - Homepage Context</t>
         </is>
       </c>
       <c r="B6" s="22" t="inlineStr"/>
@@ -2601,21 +2938,9 @@
           <t>page_view</t>
         </is>
       </c>
-      <c r="D6" s="22" t="inlineStr">
-        <is>
-          <t>search</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>select_content</t>
-        </is>
-      </c>
-      <c r="F6" s="22" t="inlineStr">
-        <is>
-          <t>account_access_intent</t>
-        </is>
-      </c>
+      <c r="D6" s="22" t="inlineStr"/>
+      <c r="E6" s="22" t="inlineStr"/>
+      <c r="F6" s="22" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
@@ -2633,26 +2958,14 @@
           <t>automatic</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="E7" s="23" t="inlineStr">
-        <is>
-          <t>recommended</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="inlineStr">
-        <is>
-          <t>custom</t>
-        </is>
-      </c>
+      <c r="D7" s="23" t="inlineStr"/>
+      <c r="E7" s="23" t="inlineStr"/>
+      <c r="F7" s="23" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>trigger</t>
+          <t>evidence_status</t>
         </is>
       </c>
       <c r="B8" s="23" t="inlineStr">
@@ -2662,29 +2975,17 @@
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Homepage load or SPA route change to the homepage.</t>
-        </is>
-      </c>
-      <c r="D8" s="23" t="inlineStr">
-        <is>
-          <t>User submits the site search form.</t>
-        </is>
-      </c>
-      <c r="E8" s="23" t="inlineStr">
-        <is>
-          <t>User clicks a consolidated navigation or content module.</t>
-        </is>
-      </c>
-      <c r="F8" s="23" t="inlineStr">
-        <is>
-          <t>User clicks the account access entry point before the login result is known.</t>
-        </is>
-      </c>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr"/>
+      <c r="E8" s="23" t="inlineStr"/>
+      <c r="F8" s="23" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>event</t>
+          <t>analysis_use</t>
         </is>
       </c>
       <c r="B9" s="23" t="inlineStr">
@@ -2694,29 +2995,17 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>page_view</t>
-        </is>
-      </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>search</t>
-        </is>
-      </c>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>select_content</t>
-        </is>
-      </c>
-      <c r="F9" s="23" t="inlineStr">
-        <is>
-          <t>account_access_intent</t>
-        </is>
-      </c>
+          <t>How many users view the homepage and from which acquisition contexts?</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr"/>
+      <c r="E9" s="23" t="inlineStr"/>
+      <c r="F9" s="23" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>page_location</t>
+          <t>trigger</t>
         </is>
       </c>
       <c r="B10" s="23" t="inlineStr">
@@ -2726,29 +3015,17 @@
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>%current_url%</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>Homepage load or SPA route change to the homepage.</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr"/>
+      <c r="E10" s="23" t="inlineStr"/>
+      <c r="F10" s="23" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>page_title</t>
+          <t>event</t>
         </is>
       </c>
       <c r="B11" s="23" t="inlineStr">
@@ -2758,29 +3035,17 @@
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>%document_title%</t>
-        </is>
-      </c>
-      <c r="D11" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E11" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>page_view</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr"/>
+      <c r="E11" s="23" t="inlineStr"/>
+      <c r="F11" s="23" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>page_referrer</t>
+          <t>page_location</t>
         </is>
       </c>
       <c r="B12" s="23" t="inlineStr">
@@ -2790,29 +3055,17 @@
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>%document_referrer%</t>
-        </is>
-      </c>
-      <c r="D12" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E12" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>%current_url%</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr"/>
+      <c r="E12" s="23" t="inlineStr"/>
+      <c r="F12" s="23" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t>page_data.template</t>
+          <t>page_title</t>
         </is>
       </c>
       <c r="B13" s="23" t="inlineStr">
@@ -2822,29 +3075,17 @@
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>homepage</t>
-        </is>
-      </c>
-      <c r="D13" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E13" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F13" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>%document_title%</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr"/>
+      <c r="E13" s="23" t="inlineStr"/>
+      <c r="F13" s="23" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t>search_term</t>
+          <t>page_referrer</t>
         </is>
       </c>
       <c r="B14" s="23" t="inlineStr">
@@ -2854,29 +3095,17 @@
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="23" t="inlineStr">
-        <is>
-          <t>%scrubbed_search_term%</t>
-        </is>
-      </c>
-      <c r="E14" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>%document_referrer%</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr"/>
+      <c r="E14" s="23" t="inlineStr"/>
+      <c r="F14" s="23" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>content_type</t>
+          <t>page_data.template</t>
         </is>
       </c>
       <c r="B15" s="23" t="inlineStr">
@@ -2886,61 +3115,37 @@
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D15" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E15" s="23" t="inlineStr">
-        <is>
-          <t>category_navigation | editorial_module | service_link</t>
-        </is>
-      </c>
-      <c r="F15" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="23" t="inlineStr">
-        <is>
-          <t>content_id</t>
-        </is>
-      </c>
-      <c r="B16" s="23" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C16" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D16" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E16" s="23" t="inlineStr">
-        <is>
-          <t>%stable_content_id%</t>
-        </is>
-      </c>
-      <c r="F16" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>homepage</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr"/>
+      <c r="E15" s="23" t="inlineStr"/>
+      <c r="F15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>J-002 - Homepage discovery - Ecommerce promotions</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr"/>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>view_promotion</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>select_promotion</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="inlineStr"/>
+      <c r="F16" s="22" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>content_name</t>
+          <t>event_classification</t>
         </is>
       </c>
       <c r="B17" s="23" t="inlineStr">
@@ -2950,29 +3155,21 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>recommended_ecommerce</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E17" s="23" t="inlineStr">
-        <is>
-          <t>%normalized_content_name%</t>
-        </is>
-      </c>
-      <c r="F17" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>recommended_ecommerce</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr"/>
+      <c r="F17" s="23" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>cta_location</t>
+          <t>evidence_status</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
@@ -2982,29 +3179,21 @@
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>inferred | medium</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E18" s="23" t="inlineStr">
-        <is>
-          <t>header | hero | body | footer</t>
-        </is>
-      </c>
-      <c r="F18" s="23" t="inlineStr">
-        <is>
-          <t>header | menu</t>
-        </is>
-      </c>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr"/>
+      <c r="F18" s="23" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>link_url</t>
+          <t>analysis_use</t>
         </is>
       </c>
       <c r="B19" s="23" t="inlineStr">
@@ -3014,29 +3203,21 @@
       </c>
       <c r="C19" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Which homepage promotions are exposed to users?</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="23" t="inlineStr">
-        <is>
-          <t>%destination_url%</t>
-        </is>
-      </c>
-      <c r="F19" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+          <t>Which exposed promotions drive clicks?</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr"/>
+      <c r="F19" s="23" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>cta_text</t>
+          <t>trigger</t>
         </is>
       </c>
       <c r="B20" s="23" t="inlineStr">
@@ -3046,29 +3227,21 @@
       </c>
       <c r="C20" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Promotion module is visible according to the agreed impression threshold.</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="23" t="inlineStr">
-        <is>
-          <t>%normalized_cta_text%</t>
-        </is>
-      </c>
+          <t>User clicks a tracked homepage promotion.</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr"/>
+      <c r="F20" s="23" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>login_status</t>
+          <t>event</t>
         </is>
       </c>
       <c r="B21" s="23" t="inlineStr">
@@ -3078,49 +3251,45 @@
       </c>
       <c r="C21" s="23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>view_promotion</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E21" s="23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="23" t="inlineStr">
-        <is>
-          <t>logged | not_logged | unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="22" t="inlineStr">
-        <is>
-          <t>J-002 - Homepage discovery - Ecommerce promotions</t>
-        </is>
-      </c>
-      <c r="B22" s="22" t="inlineStr"/>
-      <c r="C22" s="22" t="inlineStr">
-        <is>
-          <t>view_promotion</t>
-        </is>
-      </c>
-      <c r="D22" s="22" t="inlineStr">
-        <is>
           <t>select_promotion</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr"/>
-      <c r="F22" s="22" t="inlineStr"/>
+      <c r="E21" s="23" t="inlineStr"/>
+      <c r="F21" s="23" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>creative_name</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>%creative_name%</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>%creative_name%</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="inlineStr"/>
+      <c r="F22" s="23" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
         <is>
-          <t>event_classification</t>
+          <t>creative_slot</t>
         </is>
       </c>
       <c r="B23" s="23" t="inlineStr">
@@ -3130,12 +3299,12 @@
       </c>
       <c r="C23" s="23" t="inlineStr">
         <is>
-          <t>recommended_ecommerce</t>
+          <t>%creative_slot%</t>
         </is>
       </c>
       <c r="D23" s="23" t="inlineStr">
         <is>
-          <t>recommended_ecommerce</t>
+          <t>%creative_slot%</t>
         </is>
       </c>
       <c r="E23" s="23" t="inlineStr"/>
@@ -3144,7 +3313,7 @@
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
         <is>
-          <t>trigger</t>
+          <t>promotion_id</t>
         </is>
       </c>
       <c r="B24" s="23" t="inlineStr">
@@ -3154,12 +3323,12 @@
       </c>
       <c r="C24" s="23" t="inlineStr">
         <is>
-          <t>Promotion module is visible according to the agreed impression threshold.</t>
+          <t>%promotion_id%</t>
         </is>
       </c>
       <c r="D24" s="23" t="inlineStr">
         <is>
-          <t>User clicks a tracked homepage promotion.</t>
+          <t>%promotion_id%</t>
         </is>
       </c>
       <c r="E24" s="23" t="inlineStr"/>
@@ -3168,7 +3337,7 @@
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
         <is>
-          <t>event</t>
+          <t>promotion_name</t>
         </is>
       </c>
       <c r="B25" s="23" t="inlineStr">
@@ -3178,12 +3347,12 @@
       </c>
       <c r="C25" s="23" t="inlineStr">
         <is>
-          <t>view_promotion</t>
+          <t>%promotion_name%</t>
         </is>
       </c>
       <c r="D25" s="23" t="inlineStr">
         <is>
-          <t>select_promotion</t>
+          <t>%promotion_name%</t>
         </is>
       </c>
       <c r="E25" s="23" t="inlineStr"/>
@@ -3192,22 +3361,22 @@
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>currency</t>
+          <t>items</t>
         </is>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C26" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D26" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
+          <t>array&lt;object&gt;</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="inlineStr">
+        <is>
+          <t>Array&lt;Item&gt;; see items[] rows below</t>
+        </is>
+      </c>
+      <c r="D26" s="23" t="inlineStr">
+        <is>
+          <t>Array&lt;Item&gt;; see items[] rows below</t>
         </is>
       </c>
       <c r="E26" s="23" t="inlineStr"/>
@@ -3216,7 +3385,7 @@
     <row r="27">
       <c r="A27" s="23" t="inlineStr">
         <is>
-          <t>promotion_id</t>
+          <t>items[].item_id</t>
         </is>
       </c>
       <c r="B27" s="23" t="inlineStr">
@@ -3226,12 +3395,12 @@
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>%promotion_id%</t>
+          <t>%promotion_item_id%</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>%promotion_id%</t>
+          <t>%promotion_item_id%</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr"/>
@@ -3240,7 +3409,7 @@
     <row r="28">
       <c r="A28" s="23" t="inlineStr">
         <is>
-          <t>promotion_name</t>
+          <t>items[].item_name</t>
         </is>
       </c>
       <c r="B28" s="23" t="inlineStr">
@@ -3250,12 +3419,12 @@
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
-          <t>%promotion_name%</t>
+          <t>%promotion_item_name%</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
         <is>
-          <t>%promotion_name%</t>
+          <t>%promotion_item_name%</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr"/>
@@ -3264,7 +3433,7 @@
     <row r="29">
       <c r="A29" s="23" t="inlineStr">
         <is>
-          <t>creative_name</t>
+          <t>items[].affiliation</t>
         </is>
       </c>
       <c r="B29" s="23" t="inlineStr">
@@ -3272,14 +3441,14 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C29" s="23" t="inlineStr">
-        <is>
-          <t>%creative_name%</t>
-        </is>
-      </c>
-      <c r="D29" s="23" t="inlineStr">
-        <is>
-          <t>%creative_name%</t>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
         </is>
       </c>
       <c r="E29" s="23" t="inlineStr"/>
@@ -3288,7 +3457,7 @@
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
-          <t>creative_slot</t>
+          <t>items[].coupon</t>
         </is>
       </c>
       <c r="B30" s="23" t="inlineStr">
@@ -3296,14 +3465,14 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C30" s="23" t="inlineStr">
-        <is>
-          <t>%creative_slot%</t>
-        </is>
-      </c>
-      <c r="D30" s="23" t="inlineStr">
-        <is>
-          <t>%creative_slot%</t>
+      <c r="C30" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
         </is>
       </c>
       <c r="E30" s="23" t="inlineStr"/>
@@ -3312,22 +3481,22 @@
     <row r="31">
       <c r="A31" s="23" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>items[].discount</t>
         </is>
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>array&lt;object&gt;</t>
-        </is>
-      </c>
-      <c r="C31" s="23" t="inlineStr">
-        <is>
-          <t>Array&lt;Item&gt;; see items[] rows below</t>
-        </is>
-      </c>
-      <c r="D31" s="23" t="inlineStr">
-        <is>
-          <t>Array&lt;Item&gt;; see items[] rows below</t>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
         </is>
       </c>
       <c r="E31" s="23" t="inlineStr"/>
@@ -3336,22 +3505,22 @@
     <row r="32">
       <c r="A32" s="23" t="inlineStr">
         <is>
-          <t>items[].item_id</t>
+          <t>items[].index</t>
         </is>
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C32" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_item_id%</t>
-        </is>
-      </c>
-      <c r="D32" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_item_id%</t>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="C32" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D32" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
         </is>
       </c>
       <c r="E32" s="23" t="inlineStr"/>
@@ -3360,7 +3529,7 @@
     <row r="33">
       <c r="A33" s="23" t="inlineStr">
         <is>
-          <t>items[].item_name</t>
+          <t>items[].item_brand</t>
         </is>
       </c>
       <c r="B33" s="23" t="inlineStr">
@@ -3368,14 +3537,14 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C33" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_item_name%</t>
-        </is>
-      </c>
-      <c r="D33" s="23" t="inlineStr">
-        <is>
-          <t>%promotion_item_name%</t>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="inlineStr">
+        <is>
+          <t>not_available</t>
         </is>
       </c>
       <c r="E33" s="23" t="inlineStr"/>
@@ -3384,7 +3553,7 @@
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
         <is>
-          <t>items[].affiliation</t>
+          <t>items[].item_category</t>
         </is>
       </c>
       <c r="B34" s="23" t="inlineStr">
@@ -3408,7 +3577,7 @@
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>items[].coupon</t>
+          <t>items[].item_category2</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
@@ -3432,12 +3601,12 @@
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
         <is>
-          <t>items[].discount</t>
+          <t>items[].item_category3</t>
         </is>
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C36" s="24" t="inlineStr">
@@ -3456,12 +3625,12 @@
     <row r="37">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>items[].index</t>
+          <t>items[].item_category4</t>
         </is>
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>string</t>
         </is>
       </c>
       <c r="C37" s="24" t="inlineStr">
@@ -3480,7 +3649,7 @@
     <row r="38">
       <c r="A38" s="23" t="inlineStr">
         <is>
-          <t>items[].item_brand</t>
+          <t>items[].item_category5</t>
         </is>
       </c>
       <c r="B38" s="23" t="inlineStr">
@@ -3504,7 +3673,7 @@
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category</t>
+          <t>items[].item_list_id</t>
         </is>
       </c>
       <c r="B39" s="23" t="inlineStr">
@@ -3528,7 +3697,7 @@
     <row r="40">
       <c r="A40" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category2</t>
+          <t>items[].item_list_name</t>
         </is>
       </c>
       <c r="B40" s="23" t="inlineStr">
@@ -3552,7 +3721,7 @@
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category3</t>
+          <t>items[].item_variant</t>
         </is>
       </c>
       <c r="B41" s="23" t="inlineStr">
@@ -3576,7 +3745,7 @@
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category4</t>
+          <t>items[].location_id</t>
         </is>
       </c>
       <c r="B42" s="23" t="inlineStr">
@@ -3600,12 +3769,12 @@
     <row r="43">
       <c r="A43" s="23" t="inlineStr">
         <is>
-          <t>items[].item_category5</t>
+          <t>items[].price</t>
         </is>
       </c>
       <c r="B43" s="23" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>number</t>
         </is>
       </c>
       <c r="C43" s="24" t="inlineStr">
@@ -3624,22 +3793,22 @@
     <row r="44">
       <c r="A44" s="23" t="inlineStr">
         <is>
-          <t>items[].item_list_id</t>
+          <t>items[].quantity</t>
         </is>
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C44" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D44" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="C44" s="25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D44" s="25" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="E44" s="23" t="inlineStr"/>
@@ -3648,7 +3817,7 @@
     <row r="45">
       <c r="A45" s="23" t="inlineStr">
         <is>
-          <t>items[].item_list_name</t>
+          <t>items[].creative_name</t>
         </is>
       </c>
       <c r="B45" s="23" t="inlineStr">
@@ -3656,14 +3825,14 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C45" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D45" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
+      <c r="C45" s="26" t="inlineStr">
+        <is>
+          <t>event-level creative_name: %creative_name%</t>
+        </is>
+      </c>
+      <c r="D45" s="26" t="inlineStr">
+        <is>
+          <t>event-level creative_name: %creative_name%</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr"/>
@@ -3672,7 +3841,7 @@
     <row r="46">
       <c r="A46" s="23" t="inlineStr">
         <is>
-          <t>items[].item_variant</t>
+          <t>items[].creative_slot</t>
         </is>
       </c>
       <c r="B46" s="23" t="inlineStr">
@@ -3680,14 +3849,14 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C46" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D46" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>event-level creative_slot: %creative_slot%</t>
+        </is>
+      </c>
+      <c r="D46" s="26" t="inlineStr">
+        <is>
+          <t>event-level creative_slot: %creative_slot%</t>
         </is>
       </c>
       <c r="E46" s="23" t="inlineStr"/>
@@ -3696,7 +3865,7 @@
     <row r="47">
       <c r="A47" s="23" t="inlineStr">
         <is>
-          <t>items[].location_id</t>
+          <t>items[].promotion_id</t>
         </is>
       </c>
       <c r="B47" s="23" t="inlineStr">
@@ -3704,14 +3873,14 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C47" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D47" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
+      <c r="C47" s="26" t="inlineStr">
+        <is>
+          <t>event-level promotion_id: %promotion_id%</t>
+        </is>
+      </c>
+      <c r="D47" s="26" t="inlineStr">
+        <is>
+          <t>event-level promotion_id: %promotion_id%</t>
         </is>
       </c>
       <c r="E47" s="23" t="inlineStr"/>
@@ -3720,55 +3889,47 @@
     <row r="48">
       <c r="A48" s="23" t="inlineStr">
         <is>
-          <t>items[].price</t>
+          <t>items[].promotion_name</t>
         </is>
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="C48" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
-        </is>
-      </c>
-      <c r="D48" s="24" t="inlineStr">
-        <is>
-          <t>not_available</t>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>event-level promotion_name: %promotion_name%</t>
+        </is>
+      </c>
+      <c r="D48" s="26" t="inlineStr">
+        <is>
+          <t>event-level promotion_name: %promotion_name%</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr"/>
       <c r="F48" s="23" t="inlineStr"/>
     </row>
-    <row r="49">
-      <c r="A49" s="23" t="inlineStr">
-        <is>
-          <t>items[].quantity</t>
-        </is>
-      </c>
-      <c r="B49" s="23" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="C49" s="25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D49" s="25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E49" s="23" t="inlineStr"/>
-      <c r="F49" s="23" t="inlineStr"/>
+    <row r="49" ht="24" customHeight="1">
+      <c r="A49" s="22" t="inlineStr">
+        <is>
+          <t>J-003 - Homepage discovery - Site Search</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="inlineStr"/>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="D49" s="22" t="inlineStr"/>
+      <c r="E49" s="22" t="inlineStr"/>
+      <c r="F49" s="22" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="23" t="inlineStr">
         <is>
-          <t>items[].creative_name</t>
+          <t>event_classification</t>
         </is>
       </c>
       <c r="B50" s="23" t="inlineStr">
@@ -3776,23 +3937,19 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C50" s="26" t="inlineStr">
-        <is>
-          <t>event-level creative_name: %creative_name%</t>
-        </is>
-      </c>
-      <c r="D50" s="26" t="inlineStr">
-        <is>
-          <t>event-level creative_name: %creative_name%</t>
-        </is>
-      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="D50" s="23" t="inlineStr"/>
       <c r="E50" s="23" t="inlineStr"/>
       <c r="F50" s="23" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="23" t="inlineStr">
         <is>
-          <t>items[].creative_slot</t>
+          <t>evidence_status</t>
         </is>
       </c>
       <c r="B51" s="23" t="inlineStr">
@@ -3800,23 +3957,19 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C51" s="26" t="inlineStr">
-        <is>
-          <t>event-level creative_slot: %creative_slot%</t>
-        </is>
-      </c>
-      <c r="D51" s="26" t="inlineStr">
-        <is>
-          <t>event-level creative_slot: %creative_slot%</t>
-        </is>
-      </c>
+      <c r="C51" s="23" t="inlineStr">
+        <is>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D51" s="23" t="inlineStr"/>
       <c r="E51" s="23" t="inlineStr"/>
       <c r="F51" s="23" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="23" t="inlineStr">
         <is>
-          <t>items[].promotion_id</t>
+          <t>analysis_use</t>
         </is>
       </c>
       <c r="B52" s="23" t="inlineStr">
@@ -3824,23 +3977,19 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C52" s="26" t="inlineStr">
-        <is>
-          <t>event-level promotion_id: %promotion_id%</t>
-        </is>
-      </c>
-      <c r="D52" s="26" t="inlineStr">
-        <is>
-          <t>event-level promotion_id: %promotion_id%</t>
-        </is>
-      </c>
+      <c r="C52" s="23" t="inlineStr">
+        <is>
+          <t>What do users search for from the homepage?</t>
+        </is>
+      </c>
+      <c r="D52" s="23" t="inlineStr"/>
       <c r="E52" s="23" t="inlineStr"/>
       <c r="F52" s="23" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="23" t="inlineStr">
         <is>
-          <t>items[].promotion_name</t>
+          <t>trigger</t>
         </is>
       </c>
       <c r="B53" s="23" t="inlineStr">
@@ -3848,21 +3997,449 @@
           <t>string</t>
         </is>
       </c>
-      <c r="C53" s="26" t="inlineStr">
-        <is>
-          <t>event-level promotion_name: %promotion_name%</t>
-        </is>
-      </c>
-      <c r="D53" s="26" t="inlineStr">
-        <is>
-          <t>event-level promotion_name: %promotion_name%</t>
-        </is>
-      </c>
+      <c r="C53" s="23" t="inlineStr">
+        <is>
+          <t>User submits the site search form.</t>
+        </is>
+      </c>
+      <c r="D53" s="23" t="inlineStr"/>
       <c r="E53" s="23" t="inlineStr"/>
       <c r="F53" s="23" t="inlineStr"/>
     </row>
+    <row r="54">
+      <c r="A54" s="23" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B54" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C54" s="23" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="D54" s="23" t="inlineStr"/>
+      <c r="E54" s="23" t="inlineStr"/>
+      <c r="F54" s="23" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="23" t="inlineStr">
+        <is>
+          <t>search_term</t>
+        </is>
+      </c>
+      <c r="B55" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C55" s="23" t="inlineStr">
+        <is>
+          <t>%scrubbed_search_term%</t>
+        </is>
+      </c>
+      <c r="D55" s="23" t="inlineStr"/>
+      <c r="E55" s="23" t="inlineStr"/>
+      <c r="F55" s="23" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="23" t="inlineStr">
+        <is>
+          <t>page_data.template</t>
+        </is>
+      </c>
+      <c r="B56" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C56" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="23" t="inlineStr"/>
+      <c r="E56" s="23" t="inlineStr"/>
+      <c r="F56" s="23" t="inlineStr"/>
+    </row>
+    <row r="57" ht="24" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
+        <is>
+          <t>J-004 - Homepage discovery - Content Navigation Selection</t>
+        </is>
+      </c>
+      <c r="B57" s="22" t="inlineStr"/>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>select_content</t>
+        </is>
+      </c>
+      <c r="D57" s="22" t="inlineStr"/>
+      <c r="E57" s="22" t="inlineStr"/>
+      <c r="F57" s="22" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="23" t="inlineStr">
+        <is>
+          <t>event_classification</t>
+        </is>
+      </c>
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C58" s="23" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="D58" s="23" t="inlineStr"/>
+      <c r="E58" s="23" t="inlineStr"/>
+      <c r="F58" s="23" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="23" t="inlineStr">
+        <is>
+          <t>evidence_status</t>
+        </is>
+      </c>
+      <c r="B59" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C59" s="23" t="inlineStr">
+        <is>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D59" s="23" t="inlineStr"/>
+      <c r="E59" s="23" t="inlineStr"/>
+      <c r="F59" s="23" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="23" t="inlineStr">
+        <is>
+          <t>analysis_use</t>
+        </is>
+      </c>
+      <c r="B60" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C60" s="23" t="inlineStr">
+        <is>
+          <t>Which homepage modules or navigation paths drive user interest?</t>
+        </is>
+      </c>
+      <c r="D60" s="23" t="inlineStr"/>
+      <c r="E60" s="23" t="inlineStr"/>
+      <c r="F60" s="23" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="23" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="B61" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C61" s="23" t="inlineStr">
+        <is>
+          <t>User clicks a consolidated navigation or content module.</t>
+        </is>
+      </c>
+      <c r="D61" s="23" t="inlineStr"/>
+      <c r="E61" s="23" t="inlineStr"/>
+      <c r="F61" s="23" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="23" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="inlineStr">
+        <is>
+          <t>select_content</t>
+        </is>
+      </c>
+      <c r="D62" s="23" t="inlineStr"/>
+      <c r="E62" s="23" t="inlineStr"/>
+      <c r="F62" s="23" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="23" t="inlineStr">
+        <is>
+          <t>content_type</t>
+        </is>
+      </c>
+      <c r="B63" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C63" s="23" t="inlineStr">
+        <is>
+          <t>category_navigation | editorial_module | service_link</t>
+        </is>
+      </c>
+      <c r="D63" s="23" t="inlineStr"/>
+      <c r="E63" s="23" t="inlineStr"/>
+      <c r="F63" s="23" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="23" t="inlineStr">
+        <is>
+          <t>content_id</t>
+        </is>
+      </c>
+      <c r="B64" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C64" s="23" t="inlineStr">
+        <is>
+          <t>%stable_content_id%</t>
+        </is>
+      </c>
+      <c r="D64" s="23" t="inlineStr"/>
+      <c r="E64" s="23" t="inlineStr"/>
+      <c r="F64" s="23" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="23" t="inlineStr">
+        <is>
+          <t>content_name</t>
+        </is>
+      </c>
+      <c r="B65" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C65" s="23" t="inlineStr">
+        <is>
+          <t>%normalized_content_name%</t>
+        </is>
+      </c>
+      <c r="D65" s="23" t="inlineStr"/>
+      <c r="E65" s="23" t="inlineStr"/>
+      <c r="F65" s="23" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="23" t="inlineStr">
+        <is>
+          <t>cta_location</t>
+        </is>
+      </c>
+      <c r="B66" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C66" s="23" t="inlineStr">
+        <is>
+          <t>header | hero | body | footer</t>
+        </is>
+      </c>
+      <c r="D66" s="23" t="inlineStr"/>
+      <c r="E66" s="23" t="inlineStr"/>
+      <c r="F66" s="23" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="23" t="inlineStr">
+        <is>
+          <t>link_url</t>
+        </is>
+      </c>
+      <c r="B67" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C67" s="23" t="inlineStr">
+        <is>
+          <t>%destination_url%</t>
+        </is>
+      </c>
+      <c r="D67" s="23" t="inlineStr"/>
+      <c r="E67" s="23" t="inlineStr"/>
+      <c r="F67" s="23" t="inlineStr"/>
+    </row>
+    <row r="68" ht="24" customHeight="1">
+      <c r="A68" s="22" t="inlineStr">
+        <is>
+          <t>J-005 - Homepage discovery - Account Access Intent</t>
+        </is>
+      </c>
+      <c r="B68" s="22" t="inlineStr"/>
+      <c r="C68" s="22" t="inlineStr">
+        <is>
+          <t>account_access_intent</t>
+        </is>
+      </c>
+      <c r="D68" s="22" t="inlineStr"/>
+      <c r="E68" s="22" t="inlineStr"/>
+      <c r="F68" s="22" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="23" t="inlineStr">
+        <is>
+          <t>event_classification</t>
+        </is>
+      </c>
+      <c r="B69" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C69" s="23" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="D69" s="23" t="inlineStr"/>
+      <c r="E69" s="23" t="inlineStr"/>
+      <c r="F69" s="23" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="23" t="inlineStr">
+        <is>
+          <t>evidence_status</t>
+        </is>
+      </c>
+      <c r="B70" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C70" s="23" t="inlineStr">
+        <is>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D70" s="23" t="inlineStr"/>
+      <c r="E70" s="23" t="inlineStr"/>
+      <c r="F70" s="23" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="23" t="inlineStr">
+        <is>
+          <t>analysis_use</t>
+        </is>
+      </c>
+      <c r="B71" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C71" s="23" t="inlineStr">
+        <is>
+          <t>How often do users try to access the account area from the homepage?</t>
+        </is>
+      </c>
+      <c r="D71" s="23" t="inlineStr"/>
+      <c r="E71" s="23" t="inlineStr"/>
+      <c r="F71" s="23" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="23" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
+      <c r="B72" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C72" s="23" t="inlineStr">
+        <is>
+          <t>User clicks the account access entry point before the login result is known.</t>
+        </is>
+      </c>
+      <c r="D72" s="23" t="inlineStr"/>
+      <c r="E72" s="23" t="inlineStr"/>
+      <c r="F72" s="23" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="23" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B73" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C73" s="23" t="inlineStr">
+        <is>
+          <t>account_access_intent</t>
+        </is>
+      </c>
+      <c r="D73" s="23" t="inlineStr"/>
+      <c r="E73" s="23" t="inlineStr"/>
+      <c r="F73" s="23" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="23" t="inlineStr">
+        <is>
+          <t>cta_location</t>
+        </is>
+      </c>
+      <c r="B74" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C74" s="23" t="inlineStr">
+        <is>
+          <t>header | menu</t>
+        </is>
+      </c>
+      <c r="D74" s="23" t="inlineStr"/>
+      <c r="E74" s="23" t="inlineStr"/>
+      <c r="F74" s="23" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="23" t="inlineStr">
+        <is>
+          <t>cta_text</t>
+        </is>
+      </c>
+      <c r="B75" s="23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C75" s="23" t="inlineStr">
+        <is>
+          <t>%normalized_cta_text%</t>
+        </is>
+      </c>
+      <c r="D75" s="23" t="inlineStr"/>
+      <c r="E75" s="23" t="inlineStr"/>
+      <c r="F75" s="23" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:F53"/>
+  <autoFilter ref="A5:F75"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -3873,6 +4450,410 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="76" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>DataLayer Examples</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="n"/>
+      <c r="C1" s="18" t="n"/>
+      <c r="D1" s="18" t="n"/>
+      <c r="E1" s="18" t="n"/>
+      <c r="F1" s="18" t="n"/>
+      <c r="G1" s="18" t="n"/>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Complete developer examples aligned with the Event Matrix and final GA4 payload.</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="n"/>
+      <c r="C2" s="18" t="n"/>
+      <c r="D2" s="18" t="n"/>
+      <c r="E2" s="18" t="n"/>
+      <c r="F2" s="18" t="n"/>
+      <c r="G2" s="18" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Journey</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>dataLayer.push example</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>GTM and GA4 mapping</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>Implementation notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="180" customHeight="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Homepage discovery</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>page_view</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Homepage load or SPA route change to the homepage.</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>dataLayer.push({ page_data: null });
+dataLayer.push({
+  event: "page_view",
+  page_data: {
+    location: "https://example.com/",
+    title: "%document_title%",
+    template: "homepage"
+  }
+});</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>GA4 automatic collection; do not create a duplicate manual event tag.</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Avoid duplicate page_view if enhanced measurement already sends the correct event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="180" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Homepage discovery</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>view_promotion</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Promotion module is visible according to the agreed impression threshold.</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>dataLayer.push({ ecommerce: null });
+dataLayer.push({
+  event: "view_promotion",
+  ecommerce: {
+    promotion_id: "%promotion_id%",
+    promotion_name: "%promotion_name%",
+    creative_name: "%creative_name%",
+    creative_slot: "%creative_slot%",
+    items: [
+      {
+        item_id: "%promotion_item_id%",
+        item_name: "%promotion_item_name%"
+      }
+    ]
+  }
+});</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>Custom Event trigger: view_promotion
+GA4 event name: view_promotion
+ecommerce.promotion_id -&gt; promotion_id
+ecommerce.promotion_name -&gt; promotion_name
+ecommerce.creative_name -&gt; creative_name
+ecommerce.creative_slot -&gt; creative_slot
+ecommerce.items -&gt; items
+Rows in the tracking plan use official GA4 parameter names. ecommerce.* is only the GTM source object.</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>Official GA4 ecommerce event. Use one consolidated view_promotion definition and list allowed promotion values rather than one event per banner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Homepage discovery</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>select_promotion</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>User clicks a tracked homepage promotion.</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>dataLayer.push({ ecommerce: null });
+dataLayer.push({
+  event: "select_promotion",
+  ecommerce: {
+    promotion_id: "%promotion_id%",
+    promotion_name: "%promotion_name%",
+    creative_name: "%creative_name%",
+    creative_slot: "%creative_slot%",
+    items: [
+      {
+        item_id: "%promotion_item_id%",
+        item_name: "%promotion_item_name%"
+      }
+    ]
+  }
+});</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Custom Event trigger: select_promotion
+GA4 event name: select_promotion
+ecommerce.promotion_id -&gt; promotion_id
+ecommerce.promotion_name -&gt; promotion_name
+ecommerce.creative_name -&gt; creative_name
+ecommerce.creative_slot -&gt; creative_slot
+ecommerce.items -&gt; items
+Use the same promotion identifiers as view_promotion for impression-to-click analysis.</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Official GA4 ecommerce event. Keep this as an ecommerce promotion event, not a generic click event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="180" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Homepage discovery</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>search</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>User submits the site search form.</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>dataLayer.push({ event_data: null });
+dataLayer.push({
+  event: "search",
+  event_data: {
+    search_term: "%scrubbed_search_term%"
+  }
+});</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Custom Event trigger: search
+GA4 event name: search
+event_data.search_term -&gt; search_term
+event_data.page_template -&gt; page_template
+Send the official GA4 search_term parameter after PII scrubbing.</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>Use the official recommended search event instead of a custom search_submit event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="180" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Homepage discovery</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>select_content</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>User clicks a consolidated navigation or content module.</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>dataLayer.push({ event_data: null });
+dataLayer.push({
+  event: "select_content",
+  event_data: {
+    content_type: "%content_type%",
+    content_id: "%content_id%",
+    content_name: "%content_name%",
+    cta_location: "%cta_location%",
+    link_url: "%destination_url%"
+  }
+});</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>Custom Event trigger: select_content
+GA4 event name: select_content
+event_data.content_type -&gt; content_type
+event_data.content_id -&gt; content_id
+event_data.content_name -&gt; content_name
+event_data.cta_location -&gt; cta_location
+event_data.link_url -&gt; link_url
+Group similar navigation/content clicks into one select_content event with controlled values.</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Do not create one custom event per homepage link when this consolidated event is sufficient.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="180" customHeight="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Homepage discovery</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>account_access_intent</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>inferred | medium</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>User clicks the account access entry point before the login result is known.</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>dataLayer.push({ event_data: null });
+dataLayer.push({
+  event: "account_access_intent",
+  event_data: {
+    cta_location: "%cta_location%",
+    cta_text: "%normalized_cta_text%"
+  }
+});</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>Custom Event trigger: account_access_intent
+GA4 event name: account_access_intent
+event_data.cta_location -&gt; cta_location
+event_data.cta_text -&gt; cta_text
+Use the official login event only when a login actually succeeds.</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>Custom GA4 event using the project dataLayer convention. This is custom because the official login event should represent successful authentication, not an account-link click.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:G9"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Harden gated journey and screenshot evidence workflows
</commit_message>
<xml_diff>
--- a/skill/assets/ga4_tracking_plan_template.xlsx
+++ b/skill/assets/ga4_tracking_plan_template.xlsx
@@ -4864,7 +4864,7 @@
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
@@ -4942,7 +4942,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="132" customHeight="1">
+    <row r="4" ht="216" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -4980,7 +4980,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="132" customHeight="1">
+    <row r="5" ht="216" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -5018,7 +5018,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="132" customHeight="1">
+    <row r="6" ht="216" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -5056,7 +5056,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="132" customHeight="1">
+    <row r="7" ht="216" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -5094,7 +5094,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="132" customHeight="1">
+    <row r="8" ht="216" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -5132,7 +5132,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="132" customHeight="1">
+    <row r="9" ht="216" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Homepage discovery</t>
@@ -5161,12 +5161,12 @@
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>skip_allowed</t>
+          <t>capture_required</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>Skip is allowed when approved credentials or a safe test environment are unavailable.</t>
+          <t>Capture the public account entry point with a bold red rectangle around the interaction area.</t>
         </is>
       </c>
     </row>

</xml_diff>